<commit_message>
[Stage 1] Modify text struture of backlog
</commit_message>
<xml_diff>
--- a/product backlog template.xlsx
+++ b/product backlog template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="24334"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\10521\Desktop\软件工程\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lenovo\Desktop\software\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2281A449-A5C2-44A2-95A3-1D0254894067}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2160E467-B005-4346-94F2-18A841ECEBC5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2685" yWindow="2685" windowWidth="38700" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -28,15 +28,12 @@
         <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
-    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="135">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="188" uniqueCount="141">
   <si>
     <t>Story ID</t>
   </si>
@@ -1010,10 +1007,6 @@
     <phoneticPr fontId="5" type="noConversion"/>
   </si>
   <si>
-    <t>H</t>
-    <phoneticPr fontId="5" type="noConversion"/>
-  </si>
-  <si>
     <t xml:space="preserve">1. MO can fill in core job information (job title, skill requirements, weekly workload, application deadline);
 2. Published jobs are automatically displayed in the "Available Jobs" section of the system;
 3. Job information is automatically saved as a JSON file after submission;
@@ -1026,9 +1019,6 @@
     <phoneticPr fontId="5" type="noConversion"/>
   </si>
   <si>
-    <t>MO002</t>
-  </si>
-  <si>
     <t>View Applicant List for Published Jobs</t>
     <phoneticPr fontId="5" type="noConversion"/>
   </si>
@@ -1048,9 +1038,6 @@
     <phoneticPr fontId="5" type="noConversion"/>
   </si>
   <si>
-    <t>MO003</t>
-  </si>
-  <si>
     <t>Filter and Mark Applicant Status</t>
     <phoneticPr fontId="5" type="noConversion"/>
   </si>
@@ -1070,18 +1057,11 @@
     <phoneticPr fontId="5" type="noConversion"/>
   </si>
   <si>
-    <t>MO004</t>
-  </si>
-  <si>
     <t>Edit and Delete Published Jobs</t>
     <phoneticPr fontId="5" type="noConversion"/>
   </si>
   <si>
     <t>As a MO, I want to edit the details of my published jobs and take down jobs that are no longer recruiting, so that I can update job information and stop invalid applications.</t>
-    <phoneticPr fontId="5" type="noConversion"/>
-  </si>
-  <si>
-    <t>M</t>
     <phoneticPr fontId="5" type="noConversion"/>
   </si>
   <si>
@@ -1099,18 +1079,11 @@
     <phoneticPr fontId="5" type="noConversion"/>
   </si>
   <si>
-    <t>MO005</t>
-  </si>
-  <si>
     <t xml:space="preserve">	AI-assisted Screening of High-matching-rate Applicants</t>
     <phoneticPr fontId="5" type="noConversion"/>
   </si>
   <si>
     <t>As a MO, I want the system to AI-identify and highlight the high-matching-rate applicants for my jobs, so that I can focus on reviewing the most qualified applicants.</t>
-    <phoneticPr fontId="5" type="noConversion"/>
-  </si>
-  <si>
-    <t>L</t>
     <phoneticPr fontId="5" type="noConversion"/>
   </si>
   <si>
@@ -1123,6 +1096,58 @@
   </si>
   <si>
     <t xml:space="preserve">Recommendation reasons are automatically generated by AI </t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>2 story points</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>3 story points</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>1 story points</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>MO002</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>MO003</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>MO004</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>MO005</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>3 story points</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>2 story points</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>5 story points</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>High</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>Medium</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>low</t>
     <phoneticPr fontId="5" type="noConversion"/>
   </si>
 </sst>
@@ -1219,7 +1244,7 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -1234,9 +1259,6 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="176" fontId="1" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1259,9 +1281,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 主题​​">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1299,9 +1321,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
-        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -1334,26 +1356,9 @@
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -1386,26 +1391,9 @@
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
         <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1580,20 +1568,20 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:J27"/>
-  <sheetFormatPr defaultColWidth="8.875" defaultRowHeight="13.5" x14ac:dyDescent="0.15"/>
+  <sheetFormatPr defaultColWidth="8.90625" defaultRowHeight="14" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.125" style="1" customWidth="1"/>
-    <col min="2" max="2" width="16.625" style="1" customWidth="1"/>
+    <col min="1" max="1" width="9.08984375" style="1" customWidth="1"/>
+    <col min="2" max="2" width="16.6328125" style="1" customWidth="1"/>
     <col min="3" max="3" width="36" style="1" customWidth="1"/>
-    <col min="4" max="4" width="9.125" style="1"/>
-    <col min="5" max="5" width="28.375" style="1" customWidth="1"/>
-    <col min="6" max="7" width="19.875" style="1" customWidth="1"/>
-    <col min="8" max="8" width="17.125" style="1" customWidth="1"/>
-    <col min="9" max="9" width="24.875" style="1" customWidth="1"/>
-    <col min="10" max="10" width="26.375" style="1" customWidth="1"/>
+    <col min="4" max="4" width="9.08984375" style="1"/>
+    <col min="5" max="5" width="28.36328125" style="1" customWidth="1"/>
+    <col min="6" max="7" width="19.90625" style="1" customWidth="1"/>
+    <col min="8" max="8" width="17.08984375" style="1" customWidth="1"/>
+    <col min="9" max="9" width="24.90625" style="1" customWidth="1"/>
+    <col min="10" max="10" width="26.36328125" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="27" x14ac:dyDescent="0.15">
+    <row r="1" spans="1:10" ht="28" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -1625,7 +1613,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="94.5" x14ac:dyDescent="0.15">
+    <row r="2" spans="1:10" ht="98" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
         <v>53</v>
       </c>
@@ -1636,7 +1624,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:10" ht="405" x14ac:dyDescent="0.15">
+    <row r="3" spans="1:10" ht="391.5" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>12</v>
       </c>
@@ -1666,7 +1654,7 @@
         <v>46107</v>
       </c>
     </row>
-    <row r="4" spans="1:10" ht="375" x14ac:dyDescent="0.15">
+    <row r="4" spans="1:10" ht="406" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>19</v>
       </c>
@@ -1696,7 +1684,7 @@
         <v>46107</v>
       </c>
     </row>
-    <row r="5" spans="1:10" ht="409.5" x14ac:dyDescent="0.15">
+    <row r="5" spans="1:10" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
         <v>25</v>
       </c>
@@ -1726,7 +1714,7 @@
         <v>46112</v>
       </c>
     </row>
-    <row r="6" spans="1:10" ht="225" x14ac:dyDescent="0.15">
+    <row r="6" spans="1:10" ht="217.5" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
         <v>31</v>
       </c>
@@ -1756,7 +1744,7 @@
         <v>46112</v>
       </c>
     </row>
-    <row r="7" spans="1:10" ht="330" x14ac:dyDescent="0.15">
+    <row r="7" spans="1:10" ht="333.5" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
         <v>37</v>
       </c>
@@ -1786,7 +1774,7 @@
         <v>46118</v>
       </c>
     </row>
-    <row r="8" spans="1:10" ht="210" x14ac:dyDescent="0.15">
+    <row r="8" spans="1:10" ht="217.5" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
         <v>42</v>
       </c>
@@ -1816,7 +1804,7 @@
         <v>46124</v>
       </c>
     </row>
-    <row r="9" spans="1:10" ht="375" x14ac:dyDescent="0.15">
+    <row r="9" spans="1:10" ht="377" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
         <v>48</v>
       </c>
@@ -1846,7 +1834,7 @@
         <v>46132</v>
       </c>
     </row>
-    <row r="10" spans="1:10" ht="165" x14ac:dyDescent="0.15">
+    <row r="10" spans="1:10" ht="174" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
         <v>94</v>
       </c>
@@ -1856,8 +1844,8 @@
       <c r="C10" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="D10" s="3">
-        <v>1</v>
+      <c r="D10" s="3" t="s">
+        <v>138</v>
       </c>
       <c r="E10" s="3">
         <v>1</v>
@@ -1865,8 +1853,8 @@
       <c r="F10" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="G10" s="3">
-        <v>2</v>
+      <c r="G10" s="3" t="s">
+        <v>128</v>
       </c>
       <c r="H10" s="3"/>
       <c r="I10" s="3" t="s">
@@ -1874,7 +1862,7 @@
       </c>
       <c r="J10" s="3"/>
     </row>
-    <row r="11" spans="1:10" ht="150" x14ac:dyDescent="0.15">
+    <row r="11" spans="1:10" ht="145" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
         <v>95</v>
       </c>
@@ -1884,8 +1872,8 @@
       <c r="C11" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="D11" s="3">
-        <v>1</v>
+      <c r="D11" s="3" t="s">
+        <v>138</v>
       </c>
       <c r="E11" s="3">
         <v>1</v>
@@ -1893,8 +1881,8 @@
       <c r="F11" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="G11" s="3">
-        <v>3</v>
+      <c r="G11" s="3" t="s">
+        <v>129</v>
       </c>
       <c r="H11" s="3"/>
       <c r="I11" s="3" t="s">
@@ -1902,7 +1890,7 @@
       </c>
       <c r="J11" s="3"/>
     </row>
-    <row r="12" spans="1:10" ht="150" x14ac:dyDescent="0.15">
+    <row r="12" spans="1:10" ht="159.5" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
         <v>96</v>
       </c>
@@ -1912,8 +1900,8 @@
       <c r="C12" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="D12" s="3">
-        <v>1</v>
+      <c r="D12" s="3" t="s">
+        <v>138</v>
       </c>
       <c r="E12" s="3">
         <v>1</v>
@@ -1921,8 +1909,8 @@
       <c r="F12" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="G12" s="3">
-        <v>1</v>
+      <c r="G12" s="3" t="s">
+        <v>130</v>
       </c>
       <c r="H12" s="3"/>
       <c r="I12" s="3" t="s">
@@ -1930,7 +1918,7 @@
       </c>
       <c r="J12" s="3"/>
     </row>
-    <row r="13" spans="1:10" ht="135" x14ac:dyDescent="0.15">
+    <row r="13" spans="1:10" ht="130.5" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
         <v>97</v>
       </c>
@@ -1940,8 +1928,8 @@
       <c r="C13" s="3" t="s">
         <v>65</v>
       </c>
-      <c r="D13" s="3">
-        <v>1</v>
+      <c r="D13" s="3" t="s">
+        <v>138</v>
       </c>
       <c r="E13" s="3">
         <v>1</v>
@@ -1949,8 +1937,8 @@
       <c r="F13" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="G13" s="3">
-        <v>3</v>
+      <c r="G13" s="3" t="s">
+        <v>129</v>
       </c>
       <c r="H13" s="3"/>
       <c r="I13" s="3" t="s">
@@ -1958,7 +1946,7 @@
       </c>
       <c r="J13" s="3"/>
     </row>
-    <row r="14" spans="1:10" ht="150" x14ac:dyDescent="0.15">
+    <row r="14" spans="1:10" ht="145" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
         <v>98</v>
       </c>
@@ -1968,8 +1956,8 @@
       <c r="C14" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="D14" s="3">
-        <v>1</v>
+      <c r="D14" s="3" t="s">
+        <v>138</v>
       </c>
       <c r="E14" s="3">
         <v>1</v>
@@ -1977,8 +1965,8 @@
       <c r="F14" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="G14" s="3">
-        <v>3</v>
+      <c r="G14" s="3" t="s">
+        <v>129</v>
       </c>
       <c r="H14" s="3"/>
       <c r="I14" s="3" t="s">
@@ -1986,7 +1974,7 @@
       </c>
       <c r="J14" s="3"/>
     </row>
-    <row r="15" spans="1:10" ht="150" x14ac:dyDescent="0.15">
+    <row r="15" spans="1:10" ht="145" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
         <v>99</v>
       </c>
@@ -1996,8 +1984,8 @@
       <c r="C15" s="3" t="s">
         <v>71</v>
       </c>
-      <c r="D15" s="3">
-        <v>2</v>
+      <c r="D15" s="3" t="s">
+        <v>139</v>
       </c>
       <c r="E15" s="3">
         <v>1</v>
@@ -2005,8 +1993,8 @@
       <c r="F15" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="G15" s="3">
-        <v>3</v>
+      <c r="G15" s="3" t="s">
+        <v>129</v>
       </c>
       <c r="H15" s="3"/>
       <c r="I15" s="3" t="s">
@@ -2014,7 +2002,7 @@
       </c>
       <c r="J15" s="3"/>
     </row>
-    <row r="16" spans="1:10" ht="105" x14ac:dyDescent="0.15">
+    <row r="16" spans="1:10" ht="101.5" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
         <v>100</v>
       </c>
@@ -2024,8 +2012,8 @@
       <c r="C16" s="3" t="s">
         <v>74</v>
       </c>
-      <c r="D16" s="3">
-        <v>2</v>
+      <c r="D16" s="3" t="s">
+        <v>139</v>
       </c>
       <c r="E16" s="3">
         <v>1</v>
@@ -2033,8 +2021,8 @@
       <c r="F16" s="3" t="s">
         <v>75</v>
       </c>
-      <c r="G16" s="3">
-        <v>2</v>
+      <c r="G16" s="3" t="s">
+        <v>128</v>
       </c>
       <c r="H16" s="3"/>
       <c r="I16" s="3" t="s">
@@ -2042,7 +2030,7 @@
       </c>
       <c r="J16" s="3"/>
     </row>
-    <row r="17" spans="1:10" ht="135" x14ac:dyDescent="0.15">
+    <row r="17" spans="1:10" ht="130.5" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
         <v>101</v>
       </c>
@@ -2052,8 +2040,8 @@
       <c r="C17" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="D17" s="3">
-        <v>2</v>
+      <c r="D17" s="3" t="s">
+        <v>139</v>
       </c>
       <c r="E17" s="3">
         <v>1</v>
@@ -2061,8 +2049,8 @@
       <c r="F17" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="G17" s="3">
-        <v>2</v>
+      <c r="G17" s="3" t="s">
+        <v>128</v>
       </c>
       <c r="H17" s="3"/>
       <c r="I17" s="3" t="s">
@@ -2070,7 +2058,7 @@
       </c>
       <c r="J17" s="3"/>
     </row>
-    <row r="18" spans="1:10" ht="120" x14ac:dyDescent="0.15">
+    <row r="18" spans="1:10" ht="116" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
         <v>102</v>
       </c>
@@ -2080,8 +2068,8 @@
       <c r="C18" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="D18" s="3">
-        <v>2</v>
+      <c r="D18" s="3" t="s">
+        <v>139</v>
       </c>
       <c r="E18" s="3">
         <v>1</v>
@@ -2089,8 +2077,8 @@
       <c r="F18" s="3" t="s">
         <v>81</v>
       </c>
-      <c r="G18" s="3">
-        <v>3</v>
+      <c r="G18" s="3" t="s">
+        <v>129</v>
       </c>
       <c r="H18" s="3"/>
       <c r="I18" s="3" t="s">
@@ -2098,7 +2086,7 @@
       </c>
       <c r="J18" s="3"/>
     </row>
-    <row r="19" spans="1:10" ht="105" x14ac:dyDescent="0.15">
+    <row r="19" spans="1:10" ht="101.5" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
         <v>103</v>
       </c>
@@ -2108,8 +2096,8 @@
       <c r="C19" s="3" t="s">
         <v>83</v>
       </c>
-      <c r="D19" s="3">
-        <v>2</v>
+      <c r="D19" s="3" t="s">
+        <v>139</v>
       </c>
       <c r="E19" s="3">
         <v>1</v>
@@ -2117,8 +2105,8 @@
       <c r="F19" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="G19" s="3">
-        <v>3</v>
+      <c r="G19" s="3" t="s">
+        <v>129</v>
       </c>
       <c r="H19" s="3"/>
       <c r="I19" s="3" t="s">
@@ -2126,7 +2114,7 @@
       </c>
       <c r="J19" s="3"/>
     </row>
-    <row r="20" spans="1:10" ht="90" x14ac:dyDescent="0.15">
+    <row r="20" spans="1:10" ht="101.5" x14ac:dyDescent="0.25">
       <c r="A20" s="3" t="s">
         <v>104</v>
       </c>
@@ -2136,8 +2124,8 @@
       <c r="C20" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="D20" s="3">
-        <v>2</v>
+      <c r="D20" s="3" t="s">
+        <v>139</v>
       </c>
       <c r="E20" s="3">
         <v>1</v>
@@ -2145,8 +2133,8 @@
       <c r="F20" s="3" t="s">
         <v>87</v>
       </c>
-      <c r="G20" s="3">
-        <v>2</v>
+      <c r="G20" s="3" t="s">
+        <v>128</v>
       </c>
       <c r="H20" s="3"/>
       <c r="I20" s="3" t="s">
@@ -2154,7 +2142,7 @@
       </c>
       <c r="J20" s="3"/>
     </row>
-    <row r="21" spans="1:10" ht="135" x14ac:dyDescent="0.15">
+    <row r="21" spans="1:10" ht="145" x14ac:dyDescent="0.25">
       <c r="A21" s="3" t="s">
         <v>105</v>
       </c>
@@ -2164,8 +2152,8 @@
       <c r="C21" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="D21" s="3">
-        <v>3</v>
+      <c r="D21" s="3" t="s">
+        <v>140</v>
       </c>
       <c r="E21" s="3">
         <v>1</v>
@@ -2173,8 +2161,8 @@
       <c r="F21" s="3" t="s">
         <v>90</v>
       </c>
-      <c r="G21" s="3">
-        <v>2</v>
+      <c r="G21" s="3" t="s">
+        <v>128</v>
       </c>
       <c r="H21" s="3"/>
       <c r="I21" s="3" t="s">
@@ -2182,7 +2170,7 @@
       </c>
       <c r="J21" s="3"/>
     </row>
-    <row r="22" spans="1:10" ht="135" x14ac:dyDescent="0.15">
+    <row r="22" spans="1:10" ht="130.5" x14ac:dyDescent="0.25">
       <c r="A22" s="3" t="s">
         <v>106</v>
       </c>
@@ -2192,8 +2180,8 @@
       <c r="C22" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="D22" s="3">
-        <v>3</v>
+      <c r="D22" s="3" t="s">
+        <v>140</v>
       </c>
       <c r="E22" s="3">
         <v>1</v>
@@ -2201,8 +2189,8 @@
       <c r="F22" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="G22" s="3">
-        <v>3</v>
+      <c r="G22" s="3" t="s">
+        <v>129</v>
       </c>
       <c r="H22" s="3"/>
       <c r="I22" s="3" t="s">
@@ -2210,168 +2198,168 @@
       </c>
       <c r="J22" s="3"/>
     </row>
-    <row r="23" spans="1:10" ht="364.5" x14ac:dyDescent="0.15">
-      <c r="A23" s="1" t="s">
+    <row r="23" spans="1:10" ht="319" x14ac:dyDescent="0.25">
+      <c r="A23" s="3" t="s">
         <v>107</v>
       </c>
-      <c r="B23" s="1" t="s">
+      <c r="B23" s="3" t="s">
         <v>108</v>
       </c>
-      <c r="C23" s="1" t="s">
+      <c r="C23" s="3" t="s">
         <v>109</v>
       </c>
-      <c r="D23" s="1" t="s">
+      <c r="D23" s="3" t="s">
+        <v>138</v>
+      </c>
+      <c r="E23" s="3">
+        <v>1</v>
+      </c>
+      <c r="F23" s="3" t="s">
         <v>110</v>
       </c>
-      <c r="E23" s="1">
+      <c r="G23" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="H23" s="3" t="s">
+        <v>111</v>
+      </c>
+      <c r="I23" s="3">
+        <v>46101</v>
+      </c>
+      <c r="J23" s="3">
+        <v>46107</v>
+      </c>
+    </row>
+    <row r="24" spans="1:10" ht="304.5" x14ac:dyDescent="0.25">
+      <c r="A24" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="B24" s="3" t="s">
+        <v>112</v>
+      </c>
+      <c r="C24" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="D24" s="3" t="s">
+        <v>138</v>
+      </c>
+      <c r="E24" s="3">
         <v>1</v>
       </c>
-      <c r="F23" s="1" t="s">
-        <v>111</v>
-      </c>
-      <c r="G23" s="1">
-        <v>3</v>
-      </c>
-      <c r="H23" s="1" t="s">
-        <v>112</v>
-      </c>
-      <c r="I23" s="6">
-        <v>46101</v>
-      </c>
-      <c r="J23" s="6">
-        <v>46107</v>
-      </c>
-    </row>
-    <row r="24" spans="1:10" ht="310.5" x14ac:dyDescent="0.15">
-      <c r="A24" s="1" t="s">
-        <v>113</v>
-      </c>
-      <c r="B24" s="1" t="s">
+      <c r="F24" s="3" t="s">
         <v>114</v>
       </c>
-      <c r="C24" s="1" t="s">
+      <c r="G24" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="H24" s="3" t="s">
         <v>115</v>
       </c>
-      <c r="D24" s="1" t="s">
-        <v>110</v>
-      </c>
-      <c r="E24" s="1">
+      <c r="I24" s="3">
+        <v>46108</v>
+      </c>
+      <c r="J24" s="3">
+        <v>46112</v>
+      </c>
+    </row>
+    <row r="25" spans="1:10" ht="304.5" x14ac:dyDescent="0.25">
+      <c r="A25" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="B25" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="C25" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="D25" s="3" t="s">
+        <v>138</v>
+      </c>
+      <c r="E25" s="3">
         <v>1</v>
       </c>
-      <c r="F24" s="1" t="s">
-        <v>116</v>
-      </c>
-      <c r="G24" s="1">
-        <v>2</v>
-      </c>
-      <c r="H24" s="1" t="s">
-        <v>117</v>
-      </c>
-      <c r="I24" s="6">
+      <c r="F25" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="G25" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="H25" s="3" t="s">
+        <v>119</v>
+      </c>
+      <c r="I25" s="3">
         <v>46108</v>
       </c>
-      <c r="J24" s="6">
+      <c r="J25" s="3">
         <v>46112</v>
       </c>
     </row>
-    <row r="25" spans="1:10" ht="337.5" x14ac:dyDescent="0.15">
-      <c r="A25" s="1" t="s">
-        <v>118</v>
-      </c>
-      <c r="B25" s="1" t="s">
-        <v>119</v>
-      </c>
-      <c r="C25" s="1" t="s">
+    <row r="26" spans="1:10" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A26" s="3" t="s">
+        <v>133</v>
+      </c>
+      <c r="B26" s="3" t="s">
         <v>120</v>
       </c>
-      <c r="D25" s="1" t="s">
-        <v>110</v>
-      </c>
-      <c r="E25" s="1">
+      <c r="C26" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="D26" s="3" t="s">
+        <v>139</v>
+      </c>
+      <c r="E26" s="3">
         <v>1</v>
       </c>
-      <c r="F25" s="1" t="s">
-        <v>121</v>
-      </c>
-      <c r="G25" s="1">
-        <v>2</v>
-      </c>
-      <c r="H25" s="1" t="s">
+      <c r="F26" s="3" t="s">
         <v>122</v>
       </c>
-      <c r="I25" s="6">
-        <v>46108</v>
-      </c>
-      <c r="J25" s="6">
-        <v>46112</v>
-      </c>
-    </row>
-    <row r="26" spans="1:10" ht="409.5" x14ac:dyDescent="0.15">
-      <c r="A26" s="1" t="s">
+      <c r="G26" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="H26" s="3" t="s">
         <v>123</v>
       </c>
-      <c r="B26" s="1" t="s">
+      <c r="I26" s="3">
+        <v>46113</v>
+      </c>
+      <c r="J26" s="3">
+        <v>46117</v>
+      </c>
+    </row>
+    <row r="27" spans="1:10" ht="391.5" x14ac:dyDescent="0.25">
+      <c r="A27" s="3" t="s">
+        <v>134</v>
+      </c>
+      <c r="B27" s="3" t="s">
         <v>124</v>
       </c>
-      <c r="C26" s="1" t="s">
+      <c r="C27" s="3" t="s">
         <v>125</v>
       </c>
-      <c r="D26" s="1" t="s">
+      <c r="D27" s="3" t="s">
+        <v>140</v>
+      </c>
+      <c r="E27" s="3">
+        <v>1</v>
+      </c>
+      <c r="F27" s="3" t="s">
         <v>126</v>
       </c>
-      <c r="E26" s="1">
-        <v>1</v>
-      </c>
-      <c r="F26" s="1" t="s">
+      <c r="G27" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="H27" s="3" t="s">
         <v>127</v>
       </c>
-      <c r="G26" s="1">
-        <v>3</v>
-      </c>
-      <c r="H26" s="1" t="s">
-        <v>128</v>
-      </c>
-      <c r="I26" s="6">
-        <v>46113</v>
-      </c>
-      <c r="J26" s="6">
+      <c r="I27" s="3">
         <v>46117</v>
       </c>
-    </row>
-    <row r="27" spans="1:10" ht="409.5" x14ac:dyDescent="0.15">
-      <c r="A27" s="1" t="s">
-        <v>129</v>
-      </c>
-      <c r="B27" s="1" t="s">
-        <v>130</v>
-      </c>
-      <c r="C27" s="1" t="s">
-        <v>131</v>
-      </c>
-      <c r="D27" s="1" t="s">
-        <v>132</v>
-      </c>
-      <c r="E27" s="1">
-        <v>1</v>
-      </c>
-      <c r="F27" s="1" t="s">
-        <v>133</v>
-      </c>
-      <c r="G27" s="1">
-        <v>5</v>
-      </c>
-      <c r="H27" s="1" t="s">
-        <v>134</v>
-      </c>
-      <c r="I27" s="6">
-        <v>46117</v>
-      </c>
-      <c r="J27" s="6">
+      <c r="J27" s="3">
         <v>46123</v>
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="3" type="noConversion"/>
+  <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="1200" verticalDpi="1200"/>
 </worksheet>

</xml_diff>

<commit_message>
[Stage 1] Add notes for TA part.
</commit_message>
<xml_diff>
--- a/product backlog template.xlsx
+++ b/product backlog template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lenovo\Desktop\software\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2160E467-B005-4346-94F2-18A841ECEBC5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C3C2F67-7E8E-42A6-8631-1A300CCD51AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="188" uniqueCount="141">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="188" uniqueCount="153">
   <si>
     <t>Story ID</t>
   </si>
@@ -82,9 +82,6 @@
     <t>AD001</t>
   </si>
   <si>
-    <t>View Overall and Detailed Workload of All TAs</t>
-  </si>
-  <si>
     <r>
       <t>As a system admin</t>
     </r>
@@ -777,10 +774,6 @@
     <t>1. Verify the system allows saving basic info like student ID and name.
 2. Verify the system prompts and prevents saving when mandatory fields are empty.
 3. Verify data is accurately written to a local text file.</t>
-    <phoneticPr fontId="5" type="noConversion"/>
-  </si>
-  <si>
-    <t>22/03/2026</t>
     <phoneticPr fontId="5" type="noConversion"/>
   </si>
   <si>
@@ -1148,6 +1141,62 @@
   </si>
   <si>
     <t>low</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>View Overall and Detailed Workload of All TAs</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>Core conversion node of the system; must be run through in Iteration 1.</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>Forms a closed loop of business flow on the TA side.</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>Solves the pain point of time conflicts.</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>Optional field for conditional filtering.</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>Core data foundation.</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>Strongly related to the matching algorithm.</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>Core strategy to replace file uploading with links</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>Optional field for supporting highlight experiences; can be developed in Iteration 2.</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>Improves job search efficiency.</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>Enhances task management experience.</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>Fits the real-world job-seeking scenario of postgraduates.</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>Materializes the "application" action to show differentiation.</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>Lightweight implementation</t>
     <phoneticPr fontId="5" type="noConversion"/>
   </si>
 </sst>
@@ -1244,7 +1293,7 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -1259,6 +1308,9 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1615,7 +1667,7 @@
     </row>
     <row r="2" spans="1:10" ht="98" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>10</v>
@@ -1629,23 +1681,25 @@
         <v>12</v>
       </c>
       <c r="B3" s="3" t="s">
+        <v>139</v>
+      </c>
+      <c r="C3" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="D3" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="E3" s="3">
+        <v>1</v>
+      </c>
+      <c r="F3" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="E3" s="3"/>
-      <c r="F3" s="3" t="s">
+      <c r="G3" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="G3" s="3" t="s">
+      <c r="H3" s="3" t="s">
         <v>17</v>
-      </c>
-      <c r="H3" s="3" t="s">
-        <v>18</v>
       </c>
       <c r="I3" s="4">
         <v>46101</v>
@@ -1656,26 +1710,28 @@
     </row>
     <row r="4" spans="1:10" ht="406" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B4" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="C4" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="D4" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="E4" s="3">
+        <v>1</v>
+      </c>
+      <c r="F4" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="D4" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="E4" s="3"/>
-      <c r="F4" s="3" t="s">
+      <c r="G4" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="G4" s="3" t="s">
+      <c r="H4" s="3" t="s">
         <v>23</v>
-      </c>
-      <c r="H4" s="3" t="s">
-        <v>24</v>
       </c>
       <c r="I4" s="4">
         <v>46101</v>
@@ -1686,26 +1742,28 @@
     </row>
     <row r="5" spans="1:10" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="B5" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="C5" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="D5" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="E5" s="3">
+        <v>1</v>
+      </c>
+      <c r="F5" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="E5" s="3"/>
-      <c r="F5" s="3" t="s">
+      <c r="G5" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="H5" s="3" t="s">
         <v>29</v>
-      </c>
-      <c r="G5" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="H5" s="3" t="s">
-        <v>30</v>
       </c>
       <c r="I5" s="4">
         <v>46108</v>
@@ -1716,26 +1774,28 @@
     </row>
     <row r="6" spans="1:10" ht="217.5" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="B6" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="C6" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="C6" s="3" t="s">
+      <c r="D6" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="E6" s="3">
+        <v>1</v>
+      </c>
+      <c r="F6" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="D6" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="E6" s="3"/>
-      <c r="F6" s="3" t="s">
+      <c r="G6" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="G6" s="3" t="s">
+      <c r="H6" s="3" t="s">
         <v>35</v>
-      </c>
-      <c r="H6" s="3" t="s">
-        <v>36</v>
       </c>
       <c r="I6" s="4">
         <v>46108</v>
@@ -1746,26 +1806,28 @@
     </row>
     <row r="7" spans="1:10" ht="333.5" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="B7" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="C7" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="C7" s="3" t="s">
+      <c r="D7" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="E7" s="3">
+        <v>1</v>
+      </c>
+      <c r="F7" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="D7" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="E7" s="3"/>
-      <c r="F7" s="3" t="s">
+      <c r="G7" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="H7" s="3" t="s">
         <v>40</v>
-      </c>
-      <c r="G7" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="H7" s="3" t="s">
-        <v>41</v>
       </c>
       <c r="I7" s="4">
         <v>46113</v>
@@ -1776,26 +1838,28 @@
     </row>
     <row r="8" spans="1:10" ht="217.5" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="B8" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="B8" s="3" t="s">
+      <c r="C8" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="C8" s="3" t="s">
+      <c r="D8" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="D8" s="3" t="s">
+      <c r="E8" s="3">
+        <v>1</v>
+      </c>
+      <c r="F8" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="E8" s="3"/>
-      <c r="F8" s="3" t="s">
+      <c r="G8" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="H8" s="3" t="s">
         <v>46</v>
-      </c>
-      <c r="G8" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="H8" s="3" t="s">
-        <v>47</v>
       </c>
       <c r="I8" s="4">
         <v>46119</v>
@@ -1806,26 +1870,28 @@
     </row>
     <row r="9" spans="1:10" ht="377" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="B9" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="B9" s="3" t="s">
+      <c r="C9" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="C9" s="3" t="s">
+      <c r="D9" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="E9" s="3">
+        <v>1</v>
+      </c>
+      <c r="F9" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="D9" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="E9" s="3"/>
-      <c r="F9" s="3" t="s">
+      <c r="G9" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="H9" s="3" t="s">
         <v>51</v>
-      </c>
-      <c r="G9" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="H9" s="3" t="s">
-        <v>52</v>
       </c>
       <c r="I9" s="4">
         <v>46124</v>
@@ -1836,526 +1902,578 @@
     </row>
     <row r="10" spans="1:10" ht="174" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="B10" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="C10" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="C10" s="3" t="s">
+      <c r="D10" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="E10" s="3">
+        <v>1</v>
+      </c>
+      <c r="F10" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="D10" s="3" t="s">
-        <v>138</v>
-      </c>
-      <c r="E10" s="3">
-        <v>1</v>
-      </c>
-      <c r="F10" s="3" t="s">
-        <v>56</v>
-      </c>
       <c r="G10" s="3" t="s">
-        <v>128</v>
-      </c>
-      <c r="H10" s="3"/>
-      <c r="I10" s="3" t="s">
-        <v>57</v>
-      </c>
-      <c r="J10" s="3"/>
+        <v>126</v>
+      </c>
+      <c r="H10" s="3" t="s">
+        <v>144</v>
+      </c>
+      <c r="I10" s="6">
+        <v>46101</v>
+      </c>
+      <c r="J10" s="6">
+        <v>46107</v>
+      </c>
     </row>
     <row r="11" spans="1:10" ht="145" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="B11" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="E11" s="3">
+        <v>1</v>
+      </c>
+      <c r="F11" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="C11" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="D11" s="3" t="s">
-        <v>138</v>
-      </c>
-      <c r="E11" s="3">
-        <v>1</v>
-      </c>
-      <c r="F11" s="3" t="s">
-        <v>60</v>
-      </c>
       <c r="G11" s="3" t="s">
-        <v>129</v>
-      </c>
-      <c r="H11" s="3"/>
-      <c r="I11" s="3" t="s">
-        <v>57</v>
-      </c>
-      <c r="J11" s="3"/>
+        <v>127</v>
+      </c>
+      <c r="H11" s="3" t="s">
+        <v>145</v>
+      </c>
+      <c r="I11" s="6">
+        <v>46101</v>
+      </c>
+      <c r="J11" s="6">
+        <v>46107</v>
+      </c>
     </row>
     <row r="12" spans="1:10" ht="159.5" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="B12" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="D12" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="E12" s="3">
+        <v>1</v>
+      </c>
+      <c r="F12" s="3" t="s">
         <v>61</v>
       </c>
-      <c r="C12" s="3" t="s">
-        <v>62</v>
-      </c>
-      <c r="D12" s="3" t="s">
-        <v>138</v>
-      </c>
-      <c r="E12" s="3">
-        <v>1</v>
-      </c>
-      <c r="F12" s="3" t="s">
-        <v>63</v>
-      </c>
       <c r="G12" s="3" t="s">
-        <v>130</v>
-      </c>
-      <c r="H12" s="3"/>
-      <c r="I12" s="3" t="s">
-        <v>57</v>
-      </c>
-      <c r="J12" s="3"/>
+        <v>128</v>
+      </c>
+      <c r="H12" s="3" t="s">
+        <v>146</v>
+      </c>
+      <c r="I12" s="6">
+        <v>46101</v>
+      </c>
+      <c r="J12" s="6">
+        <v>46107</v>
+      </c>
     </row>
     <row r="13" spans="1:10" ht="130.5" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="B13" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="D13" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="E13" s="3">
+        <v>1</v>
+      </c>
+      <c r="F13" s="3" t="s">
         <v>64</v>
       </c>
-      <c r="C13" s="3" t="s">
-        <v>65</v>
-      </c>
-      <c r="D13" s="3" t="s">
-        <v>138</v>
-      </c>
-      <c r="E13" s="3">
-        <v>1</v>
-      </c>
-      <c r="F13" s="3" t="s">
-        <v>66</v>
-      </c>
       <c r="G13" s="3" t="s">
-        <v>129</v>
-      </c>
-      <c r="H13" s="3"/>
-      <c r="I13" s="3" t="s">
-        <v>57</v>
-      </c>
-      <c r="J13" s="3"/>
+        <v>127</v>
+      </c>
+      <c r="H13" s="3" t="s">
+        <v>142</v>
+      </c>
+      <c r="I13" s="6">
+        <v>46101</v>
+      </c>
+      <c r="J13" s="6">
+        <v>46107</v>
+      </c>
     </row>
     <row r="14" spans="1:10" ht="145" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="B14" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="D14" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="E14" s="3">
+        <v>1</v>
+      </c>
+      <c r="F14" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="C14" s="3" t="s">
-        <v>68</v>
-      </c>
-      <c r="D14" s="3" t="s">
-        <v>138</v>
-      </c>
-      <c r="E14" s="3">
-        <v>1</v>
-      </c>
-      <c r="F14" s="3" t="s">
-        <v>69</v>
-      </c>
       <c r="G14" s="3" t="s">
-        <v>129</v>
-      </c>
-      <c r="H14" s="3"/>
-      <c r="I14" s="3" t="s">
-        <v>57</v>
-      </c>
-      <c r="J14" s="3"/>
+        <v>127</v>
+      </c>
+      <c r="H14" s="3" t="s">
+        <v>141</v>
+      </c>
+      <c r="I14" s="6">
+        <v>46101</v>
+      </c>
+      <c r="J14" s="6">
+        <v>46107</v>
+      </c>
     </row>
     <row r="15" spans="1:10" ht="145" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="B15" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="C15" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="D15" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="E15" s="3">
+        <v>1</v>
+      </c>
+      <c r="F15" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="C15" s="3" t="s">
-        <v>71</v>
-      </c>
-      <c r="D15" s="3" t="s">
-        <v>139</v>
-      </c>
-      <c r="E15" s="3">
-        <v>1</v>
-      </c>
-      <c r="F15" s="3" t="s">
-        <v>72</v>
-      </c>
       <c r="G15" s="3" t="s">
-        <v>129</v>
-      </c>
-      <c r="H15" s="3"/>
-      <c r="I15" s="3" t="s">
-        <v>57</v>
-      </c>
-      <c r="J15" s="3"/>
+        <v>127</v>
+      </c>
+      <c r="H15" s="3" t="s">
+        <v>140</v>
+      </c>
+      <c r="I15" s="6">
+        <v>46108</v>
+      </c>
+      <c r="J15" s="6">
+        <v>46112</v>
+      </c>
     </row>
     <row r="16" spans="1:10" ht="101.5" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="B16" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="C16" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="D16" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="E16" s="3">
+        <v>1</v>
+      </c>
+      <c r="F16" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="C16" s="3" t="s">
-        <v>74</v>
-      </c>
-      <c r="D16" s="3" t="s">
-        <v>139</v>
-      </c>
-      <c r="E16" s="3">
-        <v>1</v>
-      </c>
-      <c r="F16" s="3" t="s">
-        <v>75</v>
-      </c>
       <c r="G16" s="3" t="s">
-        <v>128</v>
-      </c>
-      <c r="H16" s="3"/>
-      <c r="I16" s="3" t="s">
-        <v>57</v>
-      </c>
-      <c r="J16" s="3"/>
+        <v>126</v>
+      </c>
+      <c r="H16" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="I16" s="6">
+        <v>46108</v>
+      </c>
+      <c r="J16" s="6">
+        <v>46112</v>
+      </c>
     </row>
     <row r="17" spans="1:10" ht="130.5" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="B17" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="D17" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="E17" s="3">
+        <v>1</v>
+      </c>
+      <c r="F17" s="3" t="s">
         <v>76</v>
       </c>
-      <c r="C17" s="3" t="s">
-        <v>77</v>
-      </c>
-      <c r="D17" s="3" t="s">
-        <v>139</v>
-      </c>
-      <c r="E17" s="3">
-        <v>1</v>
-      </c>
-      <c r="F17" s="3" t="s">
-        <v>78</v>
-      </c>
       <c r="G17" s="3" t="s">
-        <v>128</v>
-      </c>
-      <c r="H17" s="3"/>
-      <c r="I17" s="3" t="s">
-        <v>57</v>
-      </c>
-      <c r="J17" s="3"/>
+        <v>126</v>
+      </c>
+      <c r="H17" s="3" t="s">
+        <v>147</v>
+      </c>
+      <c r="I17" s="6">
+        <v>46108</v>
+      </c>
+      <c r="J17" s="6">
+        <v>46112</v>
+      </c>
     </row>
     <row r="18" spans="1:10" ht="116" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="B18" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="C18" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="D18" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="E18" s="3">
+        <v>1</v>
+      </c>
+      <c r="F18" s="3" t="s">
         <v>79</v>
       </c>
-      <c r="C18" s="3" t="s">
-        <v>80</v>
-      </c>
-      <c r="D18" s="3" t="s">
-        <v>139</v>
-      </c>
-      <c r="E18" s="3">
-        <v>1</v>
-      </c>
-      <c r="F18" s="3" t="s">
-        <v>81</v>
-      </c>
       <c r="G18" s="3" t="s">
-        <v>129</v>
-      </c>
-      <c r="H18" s="3"/>
-      <c r="I18" s="3" t="s">
-        <v>57</v>
-      </c>
-      <c r="J18" s="3"/>
+        <v>127</v>
+      </c>
+      <c r="H18" s="3" t="s">
+        <v>148</v>
+      </c>
+      <c r="I18" s="6">
+        <v>46108</v>
+      </c>
+      <c r="J18" s="6">
+        <v>46112</v>
+      </c>
     </row>
     <row r="19" spans="1:10" ht="101.5" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="B19" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="C19" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="D19" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="E19" s="3">
+        <v>1</v>
+      </c>
+      <c r="F19" s="3" t="s">
         <v>82</v>
       </c>
-      <c r="C19" s="3" t="s">
-        <v>83</v>
-      </c>
-      <c r="D19" s="3" t="s">
-        <v>139</v>
-      </c>
-      <c r="E19" s="3">
-        <v>1</v>
-      </c>
-      <c r="F19" s="3" t="s">
-        <v>84</v>
-      </c>
       <c r="G19" s="3" t="s">
-        <v>129</v>
-      </c>
-      <c r="H19" s="3"/>
-      <c r="I19" s="3" t="s">
-        <v>57</v>
-      </c>
-      <c r="J19" s="3"/>
+        <v>127</v>
+      </c>
+      <c r="H19" s="3" t="s">
+        <v>149</v>
+      </c>
+      <c r="I19" s="6">
+        <v>46108</v>
+      </c>
+      <c r="J19" s="6">
+        <v>46112</v>
+      </c>
     </row>
     <row r="20" spans="1:10" ht="101.5" x14ac:dyDescent="0.25">
       <c r="A20" s="3" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="B20" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="C20" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="D20" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="E20" s="3">
+        <v>1</v>
+      </c>
+      <c r="F20" s="3" t="s">
         <v>85</v>
       </c>
-      <c r="C20" s="3" t="s">
-        <v>86</v>
-      </c>
-      <c r="D20" s="3" t="s">
-        <v>139</v>
-      </c>
-      <c r="E20" s="3">
-        <v>1</v>
-      </c>
-      <c r="F20" s="3" t="s">
-        <v>87</v>
-      </c>
       <c r="G20" s="3" t="s">
-        <v>128</v>
-      </c>
-      <c r="H20" s="3"/>
-      <c r="I20" s="3" t="s">
-        <v>57</v>
-      </c>
-      <c r="J20" s="3"/>
+        <v>126</v>
+      </c>
+      <c r="H20" s="3" t="s">
+        <v>150</v>
+      </c>
+      <c r="I20" s="6">
+        <v>46108</v>
+      </c>
+      <c r="J20" s="6">
+        <v>46112</v>
+      </c>
     </row>
     <row r="21" spans="1:10" ht="145" x14ac:dyDescent="0.25">
       <c r="A21" s="3" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="B21" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="C21" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="D21" s="3" t="s">
+        <v>138</v>
+      </c>
+      <c r="E21" s="3">
+        <v>1</v>
+      </c>
+      <c r="F21" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="C21" s="3" t="s">
-        <v>89</v>
-      </c>
-      <c r="D21" s="3" t="s">
-        <v>140</v>
-      </c>
-      <c r="E21" s="3">
-        <v>1</v>
-      </c>
-      <c r="F21" s="3" t="s">
-        <v>90</v>
-      </c>
       <c r="G21" s="3" t="s">
-        <v>128</v>
-      </c>
-      <c r="H21" s="3"/>
-      <c r="I21" s="3" t="s">
-        <v>57</v>
-      </c>
-      <c r="J21" s="3"/>
+        <v>126</v>
+      </c>
+      <c r="H21" s="3" t="s">
+        <v>151</v>
+      </c>
+      <c r="I21" s="6">
+        <v>46113</v>
+      </c>
+      <c r="J21" s="6">
+        <v>46119</v>
+      </c>
     </row>
     <row r="22" spans="1:10" ht="130.5" x14ac:dyDescent="0.25">
       <c r="A22" s="3" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="B22" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="C22" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="D22" s="3" t="s">
+        <v>138</v>
+      </c>
+      <c r="E22" s="3">
+        <v>1</v>
+      </c>
+      <c r="F22" s="3" t="s">
         <v>91</v>
       </c>
-      <c r="C22" s="3" t="s">
-        <v>92</v>
-      </c>
-      <c r="D22" s="3" t="s">
-        <v>140</v>
-      </c>
-      <c r="E22" s="3">
-        <v>1</v>
-      </c>
-      <c r="F22" s="3" t="s">
-        <v>93</v>
-      </c>
       <c r="G22" s="3" t="s">
-        <v>129</v>
-      </c>
-      <c r="H22" s="3"/>
-      <c r="I22" s="3" t="s">
-        <v>57</v>
-      </c>
-      <c r="J22" s="3"/>
+        <v>127</v>
+      </c>
+      <c r="H22" s="3" t="s">
+        <v>152</v>
+      </c>
+      <c r="I22" s="6">
+        <v>46113</v>
+      </c>
+      <c r="J22" s="6">
+        <v>46119</v>
+      </c>
     </row>
     <row r="23" spans="1:10" ht="319" x14ac:dyDescent="0.25">
       <c r="A23" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="B23" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="C23" s="3" t="s">
         <v>107</v>
       </c>
-      <c r="B23" s="3" t="s">
+      <c r="D23" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="E23" s="3">
+        <v>1</v>
+      </c>
+      <c r="F23" s="3" t="s">
         <v>108</v>
       </c>
-      <c r="C23" s="3" t="s">
+      <c r="G23" s="3" t="s">
+        <v>133</v>
+      </c>
+      <c r="H23" s="3" t="s">
         <v>109</v>
       </c>
-      <c r="D23" s="3" t="s">
-        <v>138</v>
-      </c>
-      <c r="E23" s="3">
-        <v>1</v>
-      </c>
-      <c r="F23" s="3" t="s">
-        <v>110</v>
-      </c>
-      <c r="G23" s="3" t="s">
-        <v>135</v>
-      </c>
-      <c r="H23" s="3" t="s">
-        <v>111</v>
-      </c>
-      <c r="I23" s="3">
+      <c r="I23" s="6">
         <v>46101</v>
       </c>
-      <c r="J23" s="3">
+      <c r="J23" s="6">
         <v>46107</v>
       </c>
     </row>
     <row r="24" spans="1:10" ht="304.5" x14ac:dyDescent="0.25">
       <c r="A24" s="3" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="B24" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="C24" s="3" t="s">
+        <v>111</v>
+      </c>
+      <c r="D24" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="E24" s="3">
+        <v>1</v>
+      </c>
+      <c r="F24" s="3" t="s">
         <v>112</v>
       </c>
-      <c r="C24" s="3" t="s">
+      <c r="G24" s="3" t="s">
+        <v>134</v>
+      </c>
+      <c r="H24" s="3" t="s">
         <v>113</v>
       </c>
-      <c r="D24" s="3" t="s">
-        <v>138</v>
-      </c>
-      <c r="E24" s="3">
-        <v>1</v>
-      </c>
-      <c r="F24" s="3" t="s">
-        <v>114</v>
-      </c>
-      <c r="G24" s="3" t="s">
-        <v>136</v>
-      </c>
-      <c r="H24" s="3" t="s">
-        <v>115</v>
-      </c>
-      <c r="I24" s="3">
-        <v>46108</v>
-      </c>
-      <c r="J24" s="3">
-        <v>46112</v>
+      <c r="I24" s="6">
+        <v>46101</v>
+      </c>
+      <c r="J24" s="6">
+        <v>46107</v>
       </c>
     </row>
     <row r="25" spans="1:10" ht="304.5" x14ac:dyDescent="0.25">
       <c r="A25" s="3" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="B25" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="C25" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="D25" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="E25" s="3">
+        <v>1</v>
+      </c>
+      <c r="F25" s="3" t="s">
         <v>116</v>
       </c>
-      <c r="C25" s="3" t="s">
+      <c r="G25" s="3" t="s">
+        <v>134</v>
+      </c>
+      <c r="H25" s="3" t="s">
         <v>117</v>
       </c>
-      <c r="D25" s="3" t="s">
-        <v>138</v>
-      </c>
-      <c r="E25" s="3">
-        <v>1</v>
-      </c>
-      <c r="F25" s="3" t="s">
-        <v>118</v>
-      </c>
-      <c r="G25" s="3" t="s">
-        <v>136</v>
-      </c>
-      <c r="H25" s="3" t="s">
-        <v>119</v>
-      </c>
-      <c r="I25" s="3">
-        <v>46108</v>
-      </c>
-      <c r="J25" s="3">
-        <v>46112</v>
+      <c r="I25" s="6">
+        <v>46101</v>
+      </c>
+      <c r="J25" s="6">
+        <v>46107</v>
       </c>
     </row>
     <row r="26" spans="1:10" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A26" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="B26" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="C26" s="3" t="s">
+        <v>119</v>
+      </c>
+      <c r="D26" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="E26" s="3">
+        <v>1</v>
+      </c>
+      <c r="F26" s="3" t="s">
+        <v>120</v>
+      </c>
+      <c r="G26" s="3" t="s">
         <v>133</v>
       </c>
-      <c r="B26" s="3" t="s">
-        <v>120</v>
-      </c>
-      <c r="C26" s="3" t="s">
+      <c r="H26" s="3" t="s">
         <v>121</v>
       </c>
-      <c r="D26" s="3" t="s">
-        <v>139</v>
-      </c>
-      <c r="E26" s="3">
-        <v>1</v>
-      </c>
-      <c r="F26" s="3" t="s">
-        <v>122</v>
-      </c>
-      <c r="G26" s="3" t="s">
-        <v>135</v>
-      </c>
-      <c r="H26" s="3" t="s">
-        <v>123</v>
-      </c>
-      <c r="I26" s="3">
-        <v>46113</v>
-      </c>
-      <c r="J26" s="3">
-        <v>46117</v>
+      <c r="I26" s="6">
+        <v>46108</v>
+      </c>
+      <c r="J26" s="6">
+        <v>46112</v>
       </c>
     </row>
     <row r="27" spans="1:10" ht="391.5" x14ac:dyDescent="0.25">
       <c r="A27" s="3" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="B27" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="C27" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="D27" s="3" t="s">
+        <v>138</v>
+      </c>
+      <c r="E27" s="3">
+        <v>1</v>
+      </c>
+      <c r="F27" s="3" t="s">
         <v>124</v>
       </c>
-      <c r="C27" s="3" t="s">
+      <c r="G27" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="H27" s="3" t="s">
         <v>125</v>
       </c>
-      <c r="D27" s="3" t="s">
-        <v>140</v>
-      </c>
-      <c r="E27" s="3">
-        <v>1</v>
-      </c>
-      <c r="F27" s="3" t="s">
-        <v>126</v>
-      </c>
-      <c r="G27" s="3" t="s">
-        <v>137</v>
-      </c>
-      <c r="H27" s="3" t="s">
-        <v>127</v>
-      </c>
-      <c r="I27" s="3">
-        <v>46117</v>
-      </c>
-      <c r="J27" s="3">
-        <v>46123</v>
+      <c r="I27" s="6">
+        <v>46113</v>
+      </c>
+      <c r="J27" s="6">
+        <v>46119</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
original version+modifications on admin
</commit_message>
<xml_diff>
--- a/product backlog template.xlsx
+++ b/product backlog template.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="181" uniqueCount="140">
   <si>
     <t>Story ID</t>
   </si>
@@ -496,6 +496,322 @@
   </si>
   <si>
     <t>Supplementary function of account management, ensure system security, handle various account abnormal situations quickly</t>
+  </si>
+  <si>
+    <t>TA001</t>
+  </si>
+  <si>
+    <t>Basic Personal Information</t>
+  </si>
+  <si>
+    <t>As a TA applicant, I want to create a basic profile in the system containing my personal information, so that the system can use it as base tags for automatic matching.</t>
+  </si>
+  <si>
+    <t>1. Verify the system allows saving basic info like student ID and name.
+2. Verify the system prompts and prevents saving when mandatory fields are empty.
+3. Verify data is accurately written to a local text file.</t>
+  </si>
+  <si>
+    <t>Core data foundation.</t>
+  </si>
+  <si>
+    <t>TA002</t>
+  </si>
+  <si>
+    <t>Undergraduate Course Grades Entry</t>
+  </si>
+  <si>
+    <t>As a TA applicant, I want to enter the core courses and grades I took during my undergraduate studies, so that the system can automatically identify if I meet the professional baseline during job matching.</t>
+  </si>
+  <si>
+    <t>1. Verify multiple undergraduate course records can be dynamically added.
+2. Verify the user can edit or delete records at any time.
+3. Verify data is accurately saved to the local data document.</t>
+  </si>
+  <si>
+    <t>Strongly related to the matching algorithm.</t>
+  </si>
+  <si>
+    <t>TA003</t>
+  </si>
+  <si>
+    <t>CV Link</t>
+  </si>
+  <si>
+    <t>As a TA applicant, I want to submit an online viewable link to my standardized CV in the system, so that the Module Organiser can comprehensively evaluate my overall academic abilities.</t>
+  </si>
+  <si>
+    <t>1. Verify the system provides a text box and validates the URL format.
+2. Verify this field is mandatory.
+3. Verify it is saved as plain text and displayed as a clickable hyperlink on the MO's side.</t>
+  </si>
+  <si>
+    <t>Core strategy to replace file uploading with links</t>
+  </si>
+  <si>
+    <t>TA004</t>
+  </si>
+  <si>
+    <t>Job Overview and Timetable</t>
+  </si>
+  <si>
+    <t>As a TA applicant, I want to browse all open positions for the current semester and see the start/end dates and full timetable, so that I can understand job opportunities and judge time conflicts.</t>
+  </si>
+  <si>
+    <t>1. Verify only current semester jobs are displayed.
+2. Verify clear display of MO, start/end dates, and timetable.
+3. Verify data is read and rendered from plain text files.</t>
+  </si>
+  <si>
+    <t>Solves the pain point of time conflicts.</t>
+  </si>
+  <si>
+    <t>TA005</t>
+  </si>
+  <si>
+    <t>Application Status Dashboard</t>
+  </si>
+  <si>
+    <t>As a TA applicant, I want to view the real-time review status of all historical applications in a dashboard, so that I can keep track of the progress at any time.</t>
+  </si>
+  <si>
+    <t>1. Verify historical applications are read and filtered by TA ID.
+2. Verify clear display of module, time, and status.
+3. Verify the frontend status updates synchronously with local data.</t>
+  </si>
+  <si>
+    <t>Forms a closed loop of business flow on the TA side.</t>
+  </si>
+  <si>
+    <t>TA006</t>
+  </si>
+  <si>
+    <t>One-Click Application &amp; Data Association</t>
+  </si>
+  <si>
+    <t>As a TA applicant, I want to click a submit button to apply for the job with my profile and statement together, so that I can efficiently and standardly complete the entire application process.</t>
+  </si>
+  <si>
+    <t>1. Verify the anti-duplicate submission mechanism.
+2. Verify TA ID, Job ID, and statement are packaged into one application record.
+3. Verify data is appended and written into a plain text file.</t>
+  </si>
+  <si>
+    <t>Core conversion node of the system; must be run through in Iteration 1.</t>
+  </si>
+  <si>
+    <t>TA007</t>
+  </si>
+  <si>
+    <t>Language Proficiency Details</t>
+  </si>
+  <si>
+    <t>As a TA applicant, I want to fill in my language exam scores, so that the system can use them as quantitative features for matching weight calculations.</t>
+  </si>
+  <si>
+    <t>1. Verify the system provides a language type drop-down menu and score input.
+2. Verify it is written to a local data document in CSV or JSON format.</t>
+  </si>
+  <si>
+    <t>Optional field for conditional filtering.</t>
+  </si>
+  <si>
+    <t>TA008</t>
+  </si>
+  <si>
+    <t>Supplementary Proof Materials Link</t>
+  </si>
+  <si>
+    <t>As a TA applicant, I want to submit a cloud drive link containing my additional proof documents in the system, so that I can provide factual support for specific statements in my CV.</t>
+  </si>
+  <si>
+    <t>1. Verify the system provides a link input box and a short remark input box.
+2. Verify this field is optional.
+3. Verify data is successfully saved to local CSV/JSON.</t>
+  </si>
+  <si>
+    <t>Optional field for supporting highlight experiences; can be developed in Iteration 2.</t>
+  </si>
+  <si>
+    <t>TA009</t>
+  </si>
+  <si>
+    <t>Filtered by Module Name</t>
+  </si>
+  <si>
+    <t>As a TA applicant, I want to search the current job list by entering a "module name", so that I can quickly locate courses relevant to my major.</t>
+  </si>
+  <si>
+    <t>1. Verify a text search box is provided.
+2. Verify support for fuzzy matching of module names.
+3. Verify friendly prompts when there are no results.</t>
+  </si>
+  <si>
+    <t>Improves job search efficiency.</t>
+  </si>
+  <si>
+    <t>TA010</t>
+  </si>
+  <si>
+    <t>Filtered by Deadline</t>
+  </si>
+  <si>
+    <t>As a TA applicant, I want to sort by "application deadline" and distinguish between open and closed positions, so that I can prioritize applications for jobs that are about to close.</t>
+  </si>
+  <si>
+    <t>1. Verify support for ascending sorting by deadline.
+2. Verify graying out and disabling the apply button for closed positions.</t>
+  </si>
+  <si>
+    <t>Enhances task management experience.</t>
+  </si>
+  <si>
+    <t>TA011</t>
+  </si>
+  <si>
+    <t>Filtered by MO Name</t>
+  </si>
+  <si>
+    <t>As a TA applicant, I want to filter jobs by the "MO's name", so that I can prioritize applying for courses taught by a supervisor I am familiar with.</t>
+  </si>
+  <si>
+    <t>1. Verify an MO filtering drop-down or search is provided.
+2. Verify results refresh in real-time to show only that MO's modules.</t>
+  </si>
+  <si>
+    <t>Fits the real-world job-seeking scenario of postgraduates.</t>
+  </si>
+  <si>
+    <t>TA012</t>
+  </si>
+  <si>
+    <t>Application Statement</t>
+  </si>
+  <si>
+    <t>As a TA applicant, I want to write a dedicated application statement when applying for a specific position, so that I can precisely explain to the MO why I am a match for this course.</t>
+  </si>
+  <si>
+    <t>1. Verify a text box pops up for writing during application.
+2. Verify there is a word limit and it is optional.
+3. Verify support for special characters and correct writing to plain text files.</t>
+  </si>
+  <si>
+    <t>Materializes the "application" action to show differentiation.</t>
+  </si>
+  <si>
+    <t>TA013</t>
+  </si>
+  <si>
+    <t>Status Update Login Pop-up</t>
+  </si>
+  <si>
+    <t>As a TA applicant, I want the system to automatically pop up a notification upon login if there are status updates, so that I can be informed of the most important admission results immediately.</t>
+  </si>
+  <si>
+    <t>1. Verify the system identifies "unread" status updates.
+2. Verify a pop-up triggers upon logging into the homepage.
+3. Verify it is marked as read after the pop-up is closed.</t>
+  </si>
+  <si>
+    <t>Lightweight implementation</t>
+  </si>
+  <si>
+    <t>MO001</t>
+  </si>
+  <si>
+    <t>Publish TA Recruitment Jobs</t>
+  </si>
+  <si>
+    <t>As a MO, I want to publish TA recruitment jobs with detailed information, so that eligible TA applicants can browse and apply for the relevant jobs.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. MO can fill in core job information (job title, skill requirements, weekly workload, application deadline);
+2. Published jobs are automatically displayed in the "Available Jobs" section of the system;
+3. Job information is automatically saved as a JSON file after submission;
+4. Only the publishing MO can edit their own jobs, and administrators can view all MO-published jobs.
+</t>
+  </si>
+  <si>
+    <t>Naming rule for storage files: MO_JobID_PublishDate.json;</t>
+  </si>
+  <si>
+    <t>MO002</t>
+  </si>
+  <si>
+    <t>View Applicant List for Published Jobs</t>
+  </si>
+  <si>
+    <t>As a MO, I want to view a complete list of applicants for the jobs I published, so that I can quickly get an overview of all applicants for my jobs.</t>
+  </si>
+  <si>
+    <t>1. After logging in, MO can only view applicants for their own published jobs, not for other MOs' jobs;
+2. The list displays the following fields: Applicant ID, Name, Application Time, Core Skill Tags, Application Status;
+3. Clicking the applicant's name jumps to the CV detail page;
+4. The list supports filtering by application status (Pending Review/Approved/Rejected).</t>
+  </si>
+  <si>
+    <t>Applicant skill tags extract core keywords from TA resumes;</t>
+  </si>
+  <si>
+    <t>MO003</t>
+  </si>
+  <si>
+    <t>Filter and Mark Applicant Status</t>
+  </si>
+  <si>
+    <t>As a MO, I want to mark applicants' status as "Approved"/"Rejected"/"Pending Interview" for the jobs I published, so that I can manage the recruitment review process and notify applicants of the results.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. MO can mark the status of each applicant individually, and the status is automatically synced to the applicant's system account;
+2. After marking as "Approved"/"Rejected", the system automatically generates a status notification and saves it to the applicant's notification file;
+3. Marking records are automatically saved with Marked By, Mark Time and Status for traceability;
+</t>
+  </si>
+  <si>
+    <t>Status marking data is stored in JSON format and associated with Job ID-Applicant ID;</t>
+  </si>
+  <si>
+    <t>MO004</t>
+  </si>
+  <si>
+    <t>Edit and Delete Published Jobs</t>
+  </si>
+  <si>
+    <t>As a MO, I want to edit the details of my published jobs and take down jobs that are no longer recruiting, so that I can update job information and stop invalid applications.</t>
+  </si>
+  <si>
+    <t>1. MO can edit all job information before the application deadline, and the edited content is automatically updated in the system display;
+2. MO can take down jobs at any time, and the taken-down jobs are hidden from the "Available Jobs" section and no longer accept new applications;
+3. The applicant list of taken-down jobs can still be viewed and managed normally;
+4. All edit/take-down operations are logged with Operator, Time and Operation Type;
+5. Jobs are automatically marked as "Closed" after the deadline and cannot be edited or republished.</t>
+  </si>
+  <si>
+    <t>1. Edit operations only modify the original job CSV file without generating new files;
+2. Take-down status is stored in the JSON configuration file of job information;
+3. Deadline automatic validation is triggered regularly by the system.</t>
+  </si>
+  <si>
+    <t>MO005</t>
+  </si>
+  <si>
+    <t xml:space="preserve">	AI-assisted Screening of High-matching-rate Applicants</t>
+  </si>
+  <si>
+    <t>As a MO, I want the system to AI-identify and highlight the high-matching-rate applicants for my jobs, so that I can focus on reviewing the most qualified applicants.</t>
+  </si>
+  <si>
+    <t>1. AI automatically screens out high-matching-rate applicants for the job based on the matching rate and displays them in a separate section;
+2. The high-matching-rate threshold (30%) can be manually adjusted by MO;
+3. Highlight display includes Matching Rate, Core Matched Skills and Recommendation Reasons;
+4. AI recommendation results can be refreshed and support excluding specified applicants;
+5. Recommendation results do not affect MO's manual screening and are only for auxiliary reference.</t>
+  </si>
+  <si>
+    <t>5 story points</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Recommendation reasons are automatically generated by AI </t>
   </si>
 </sst>
 </file>
@@ -509,13 +825,26 @@
     <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="176" formatCode="yyyy/m/d;@"/>
   </numFmts>
-  <fonts count="21">
+  <fonts count="23">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="宋体"/>
       <charset val="134"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
     </font>
     <font>
       <sz val="11"/>
@@ -1001,136 +1330,136 @@
     <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="6" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="19" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="21" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -1138,16 +1467,19 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="27" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="176" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="176" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1499,7 +1831,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:J27"/>
+  <dimension ref="A1:J26"/>
   <sheetFormatPr defaultColWidth="8.90909090909091" defaultRowHeight="14"/>
   <cols>
     <col min="1" max="1" width="9.09090909090909" style="1" customWidth="1"/>
@@ -1507,9 +1839,8 @@
     <col min="3" max="3" width="36" style="1" customWidth="1"/>
     <col min="4" max="4" width="9.09090909090909" style="1"/>
     <col min="5" max="5" width="28.3636363636364" style="1" customWidth="1"/>
-    <col min="6" max="6" width="33.9090909090909" style="1" customWidth="1"/>
-    <col min="7" max="7" width="19.9090909090909" style="1" customWidth="1"/>
-    <col min="8" max="8" width="28.6363636363636" style="1" customWidth="1"/>
+    <col min="6" max="7" width="19.9090909090909" style="1" customWidth="1"/>
+    <col min="8" max="8" width="17.0909090909091" style="1" customWidth="1"/>
     <col min="9" max="9" width="24.9090909090909" style="1" customWidth="1"/>
     <col min="10" max="10" width="26.3636363636364" style="1" customWidth="1"/>
   </cols>
@@ -1557,7 +1888,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="3" ht="232" spans="1:10">
+    <row r="3" ht="409.5" spans="1:10">
       <c r="A3" s="4" t="s">
         <v>13</v>
       </c>
@@ -1589,7 +1920,7 @@
         <v>46107</v>
       </c>
     </row>
-    <row r="4" ht="217.5" spans="1:10">
+    <row r="4" ht="377" spans="1:10">
       <c r="A4" s="4" t="s">
         <v>20</v>
       </c>
@@ -1621,7 +1952,7 @@
         <v>46132</v>
       </c>
     </row>
-    <row r="5" ht="275.5" spans="1:10">
+    <row r="5" ht="409.5" spans="1:10">
       <c r="A5" s="4" t="s">
         <v>25</v>
       </c>
@@ -1653,7 +1984,7 @@
         <v>46112</v>
       </c>
     </row>
-    <row r="6" ht="130.5" spans="1:10">
+    <row r="6" ht="217.5" spans="1:10">
       <c r="A6" s="4" t="s">
         <v>32</v>
       </c>
@@ -1685,7 +2016,7 @@
         <v>46112</v>
       </c>
     </row>
-    <row r="7" ht="174" spans="1:10">
+    <row r="7" ht="333.5" spans="1:10">
       <c r="A7" s="4" t="s">
         <v>38</v>
       </c>
@@ -1717,7 +2048,7 @@
         <v>46118</v>
       </c>
     </row>
-    <row r="8" ht="130.5" spans="1:10">
+    <row r="8" ht="217.5" spans="1:10">
       <c r="A8" s="4" t="s">
         <v>43</v>
       </c>
@@ -1749,233 +2080,581 @@
         <v>46124</v>
       </c>
     </row>
-    <row r="9" ht="14.5" spans="1:10">
-      <c r="A9" s="4"/>
-      <c r="B9" s="4"/>
-      <c r="C9" s="4"/>
-      <c r="D9" s="4"/>
-      <c r="E9" s="4"/>
-      <c r="F9" s="4"/>
-      <c r="G9" s="4"/>
-      <c r="H9" s="4"/>
-      <c r="I9" s="5"/>
-      <c r="J9" s="5"/>
+    <row r="9" ht="174" spans="1:10">
+      <c r="A9" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="B9" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="C9" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="D9" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="E9" s="6">
+        <v>1</v>
+      </c>
+      <c r="F9" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="G9" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="H9" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="I9" s="7">
+        <v>46101</v>
+      </c>
+      <c r="J9" s="7">
+        <v>46107</v>
+      </c>
     </row>
-    <row r="10" ht="14.5" spans="1:10">
-      <c r="A10" s="4"/>
-      <c r="B10" s="4"/>
-      <c r="C10" s="4"/>
-      <c r="D10" s="4"/>
-      <c r="E10" s="4"/>
-      <c r="F10" s="4"/>
-      <c r="G10" s="4"/>
-      <c r="H10" s="4"/>
-      <c r="I10" s="6"/>
-      <c r="J10" s="6"/>
+    <row r="10" ht="145" spans="1:10">
+      <c r="A10" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="B10" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="C10" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="D10" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="E10" s="6">
+        <v>1</v>
+      </c>
+      <c r="F10" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="G10" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="H10" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="I10" s="7">
+        <v>46101</v>
+      </c>
+      <c r="J10" s="7">
+        <v>46107</v>
+      </c>
     </row>
-    <row r="11" ht="14.5" spans="1:10">
-      <c r="A11" s="4"/>
-      <c r="B11" s="4"/>
-      <c r="C11" s="4"/>
-      <c r="D11" s="4"/>
-      <c r="E11" s="4"/>
-      <c r="F11" s="4"/>
-      <c r="G11" s="4"/>
-      <c r="H11" s="4"/>
-      <c r="I11" s="6"/>
-      <c r="J11" s="6"/>
+    <row r="11" ht="159.5" spans="1:10">
+      <c r="A11" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="B11" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="C11" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="D11" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="E11" s="6">
+        <v>1</v>
+      </c>
+      <c r="F11" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="G11" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="H11" s="6" t="s">
+        <v>63</v>
+      </c>
+      <c r="I11" s="7">
+        <v>46101</v>
+      </c>
+      <c r="J11" s="7">
+        <v>46107</v>
+      </c>
     </row>
-    <row r="12" ht="14.5" spans="1:10">
-      <c r="A12" s="4"/>
-      <c r="B12" s="4"/>
-      <c r="C12" s="4"/>
-      <c r="D12" s="4"/>
-      <c r="E12" s="4"/>
-      <c r="F12" s="4"/>
-      <c r="G12" s="4"/>
-      <c r="H12" s="4"/>
-      <c r="I12" s="6"/>
-      <c r="J12" s="6"/>
+    <row r="12" ht="130.5" spans="1:10">
+      <c r="A12" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="B12" s="6" t="s">
+        <v>65</v>
+      </c>
+      <c r="C12" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="D12" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="E12" s="6">
+        <v>1</v>
+      </c>
+      <c r="F12" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="G12" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="H12" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="I12" s="7">
+        <v>46101</v>
+      </c>
+      <c r="J12" s="7">
+        <v>46107</v>
+      </c>
     </row>
-    <row r="13" ht="14.5" spans="1:10">
-      <c r="A13" s="4"/>
-      <c r="B13" s="4"/>
-      <c r="C13" s="4"/>
-      <c r="D13" s="4"/>
-      <c r="E13" s="4"/>
-      <c r="F13" s="4"/>
-      <c r="G13" s="4"/>
-      <c r="H13" s="4"/>
-      <c r="I13" s="6"/>
-      <c r="J13" s="6"/>
+    <row r="13" ht="145" spans="1:10">
+      <c r="A13" s="6" t="s">
+        <v>69</v>
+      </c>
+      <c r="B13" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="C13" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="D13" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="E13" s="6">
+        <v>1</v>
+      </c>
+      <c r="F13" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="G13" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="H13" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="I13" s="7">
+        <v>46101</v>
+      </c>
+      <c r="J13" s="7">
+        <v>46107</v>
+      </c>
     </row>
-    <row r="14" ht="14.5" spans="1:10">
-      <c r="A14" s="4"/>
-      <c r="B14" s="4"/>
-      <c r="C14" s="4"/>
-      <c r="D14" s="4"/>
-      <c r="E14" s="4"/>
-      <c r="F14" s="4"/>
-      <c r="G14" s="4"/>
-      <c r="H14" s="4"/>
-      <c r="I14" s="6"/>
-      <c r="J14" s="6"/>
+    <row r="14" ht="145" spans="1:10">
+      <c r="A14" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="B14" s="6" t="s">
+        <v>75</v>
+      </c>
+      <c r="C14" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="D14" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="E14" s="6">
+        <v>1</v>
+      </c>
+      <c r="F14" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="G14" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="H14" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="I14" s="7">
+        <v>46108</v>
+      </c>
+      <c r="J14" s="7">
+        <v>46112</v>
+      </c>
     </row>
-    <row r="15" ht="14.5" spans="1:10">
-      <c r="A15" s="4"/>
-      <c r="B15" s="4"/>
-      <c r="C15" s="4"/>
-      <c r="D15" s="4"/>
-      <c r="E15" s="4"/>
-      <c r="F15" s="4"/>
-      <c r="G15" s="4"/>
-      <c r="H15" s="4"/>
-      <c r="I15" s="6"/>
-      <c r="J15" s="6"/>
+    <row r="15" ht="101.5" spans="1:10">
+      <c r="A15" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="B15" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="C15" s="6" t="s">
+        <v>81</v>
+      </c>
+      <c r="D15" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="E15" s="6">
+        <v>1</v>
+      </c>
+      <c r="F15" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="G15" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="H15" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="I15" s="7">
+        <v>46108</v>
+      </c>
+      <c r="J15" s="7">
+        <v>46112</v>
+      </c>
     </row>
-    <row r="16" ht="14.5" spans="1:10">
-      <c r="A16" s="4"/>
-      <c r="B16" s="4"/>
-      <c r="C16" s="4"/>
-      <c r="D16" s="4"/>
-      <c r="E16" s="4"/>
-      <c r="F16" s="4"/>
-      <c r="G16" s="4"/>
-      <c r="H16" s="4"/>
-      <c r="I16" s="6"/>
-      <c r="J16" s="6"/>
+    <row r="16" ht="130.5" spans="1:10">
+      <c r="A16" s="6" t="s">
+        <v>84</v>
+      </c>
+      <c r="B16" s="6" t="s">
+        <v>85</v>
+      </c>
+      <c r="C16" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="D16" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="E16" s="6">
+        <v>1</v>
+      </c>
+      <c r="F16" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="G16" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="H16" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="I16" s="7">
+        <v>46108</v>
+      </c>
+      <c r="J16" s="7">
+        <v>46112</v>
+      </c>
     </row>
-    <row r="17" ht="14.5" spans="1:10">
-      <c r="A17" s="4"/>
-      <c r="B17" s="4"/>
-      <c r="C17" s="4"/>
-      <c r="D17" s="4"/>
-      <c r="E17" s="4"/>
-      <c r="F17" s="4"/>
-      <c r="G17" s="4"/>
-      <c r="H17" s="4"/>
-      <c r="I17" s="6"/>
-      <c r="J17" s="6"/>
+    <row r="17" ht="116" spans="1:10">
+      <c r="A17" s="6" t="s">
+        <v>89</v>
+      </c>
+      <c r="B17" s="6" t="s">
+        <v>90</v>
+      </c>
+      <c r="C17" s="6" t="s">
+        <v>91</v>
+      </c>
+      <c r="D17" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="E17" s="6">
+        <v>1</v>
+      </c>
+      <c r="F17" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="G17" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="H17" s="6" t="s">
+        <v>93</v>
+      </c>
+      <c r="I17" s="7">
+        <v>46108</v>
+      </c>
+      <c r="J17" s="7">
+        <v>46112</v>
+      </c>
     </row>
-    <row r="18" ht="14.5" spans="1:10">
-      <c r="A18" s="4"/>
-      <c r="B18" s="4"/>
-      <c r="C18" s="4"/>
-      <c r="D18" s="4"/>
-      <c r="E18" s="4"/>
-      <c r="F18" s="4"/>
-      <c r="G18" s="4"/>
-      <c r="H18" s="4"/>
-      <c r="I18" s="6"/>
-      <c r="J18" s="6"/>
+    <row r="18" ht="101.5" spans="1:10">
+      <c r="A18" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="B18" s="6" t="s">
+        <v>95</v>
+      </c>
+      <c r="C18" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="D18" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="E18" s="6">
+        <v>1</v>
+      </c>
+      <c r="F18" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="G18" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="H18" s="6" t="s">
+        <v>98</v>
+      </c>
+      <c r="I18" s="7">
+        <v>46108</v>
+      </c>
+      <c r="J18" s="7">
+        <v>46112</v>
+      </c>
     </row>
-    <row r="19" ht="14.5" spans="1:10">
-      <c r="A19" s="4"/>
-      <c r="B19" s="4"/>
-      <c r="C19" s="4"/>
-      <c r="D19" s="4"/>
-      <c r="E19" s="4"/>
-      <c r="F19" s="4"/>
-      <c r="G19" s="4"/>
-      <c r="H19" s="4"/>
-      <c r="I19" s="6"/>
-      <c r="J19" s="6"/>
+    <row r="19" ht="101.5" spans="1:10">
+      <c r="A19" s="6" t="s">
+        <v>99</v>
+      </c>
+      <c r="B19" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="C19" s="6" t="s">
+        <v>101</v>
+      </c>
+      <c r="D19" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="E19" s="6">
+        <v>1</v>
+      </c>
+      <c r="F19" s="6" t="s">
+        <v>102</v>
+      </c>
+      <c r="G19" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="H19" s="6" t="s">
+        <v>103</v>
+      </c>
+      <c r="I19" s="7">
+        <v>46108</v>
+      </c>
+      <c r="J19" s="7">
+        <v>46112</v>
+      </c>
     </row>
-    <row r="20" ht="14.5" spans="1:10">
-      <c r="A20" s="4"/>
-      <c r="B20" s="4"/>
-      <c r="C20" s="4"/>
-      <c r="D20" s="4"/>
-      <c r="E20" s="4"/>
-      <c r="F20" s="4"/>
-      <c r="G20" s="4"/>
-      <c r="H20" s="4"/>
-      <c r="I20" s="6"/>
-      <c r="J20" s="6"/>
+    <row r="20" ht="145" spans="1:10">
+      <c r="A20" s="6" t="s">
+        <v>104</v>
+      </c>
+      <c r="B20" s="6" t="s">
+        <v>105</v>
+      </c>
+      <c r="C20" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="D20" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="E20" s="6">
+        <v>1</v>
+      </c>
+      <c r="F20" s="6" t="s">
+        <v>107</v>
+      </c>
+      <c r="G20" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="H20" s="6" t="s">
+        <v>108</v>
+      </c>
+      <c r="I20" s="7">
+        <v>46113</v>
+      </c>
+      <c r="J20" s="7">
+        <v>46119</v>
+      </c>
     </row>
-    <row r="21" ht="14.5" spans="1:10">
-      <c r="A21" s="4"/>
-      <c r="B21" s="4"/>
-      <c r="C21" s="4"/>
-      <c r="D21" s="4"/>
-      <c r="E21" s="4"/>
-      <c r="F21" s="4"/>
-      <c r="G21" s="4"/>
-      <c r="H21" s="4"/>
-      <c r="I21" s="6"/>
-      <c r="J21" s="6"/>
+    <row r="21" ht="130.5" spans="1:10">
+      <c r="A21" s="6" t="s">
+        <v>109</v>
+      </c>
+      <c r="B21" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="C21" s="6" t="s">
+        <v>111</v>
+      </c>
+      <c r="D21" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="E21" s="6">
+        <v>1</v>
+      </c>
+      <c r="F21" s="6" t="s">
+        <v>112</v>
+      </c>
+      <c r="G21" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="H21" s="6" t="s">
+        <v>113</v>
+      </c>
+      <c r="I21" s="7">
+        <v>46113</v>
+      </c>
+      <c r="J21" s="7">
+        <v>46119</v>
+      </c>
     </row>
-    <row r="22" ht="14.5" spans="1:10">
-      <c r="A22" s="4"/>
-      <c r="B22" s="4"/>
-      <c r="C22" s="4"/>
-      <c r="D22" s="4"/>
-      <c r="E22" s="4"/>
-      <c r="F22" s="4"/>
-      <c r="G22" s="4"/>
-      <c r="H22" s="4"/>
-      <c r="I22" s="6"/>
-      <c r="J22" s="6"/>
+    <row r="22" ht="319" spans="1:10">
+      <c r="A22" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="B22" s="6" t="s">
+        <v>115</v>
+      </c>
+      <c r="C22" s="6" t="s">
+        <v>116</v>
+      </c>
+      <c r="D22" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="E22" s="6">
+        <v>1</v>
+      </c>
+      <c r="F22" s="6" t="s">
+        <v>117</v>
+      </c>
+      <c r="G22" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="H22" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="I22" s="7">
+        <v>46101</v>
+      </c>
+      <c r="J22" s="7">
+        <v>46107</v>
+      </c>
     </row>
-    <row r="23" ht="14.5" spans="1:10">
-      <c r="A23" s="4"/>
-      <c r="B23" s="4"/>
-      <c r="C23" s="4"/>
-      <c r="D23" s="4"/>
-      <c r="E23" s="4"/>
-      <c r="F23" s="4"/>
-      <c r="G23" s="4"/>
-      <c r="H23" s="4"/>
-      <c r="I23" s="6"/>
-      <c r="J23" s="6"/>
+    <row r="23" ht="304.5" spans="1:10">
+      <c r="A23" s="6" t="s">
+        <v>119</v>
+      </c>
+      <c r="B23" s="6" t="s">
+        <v>120</v>
+      </c>
+      <c r="C23" s="6" t="s">
+        <v>121</v>
+      </c>
+      <c r="D23" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="E23" s="6">
+        <v>1</v>
+      </c>
+      <c r="F23" s="6" t="s">
+        <v>122</v>
+      </c>
+      <c r="G23" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="H23" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="I23" s="7">
+        <v>46101</v>
+      </c>
+      <c r="J23" s="7">
+        <v>46107</v>
+      </c>
     </row>
-    <row r="24" ht="14.5" spans="1:10">
-      <c r="A24" s="4"/>
-      <c r="B24" s="4"/>
-      <c r="C24" s="4"/>
-      <c r="D24" s="4"/>
-      <c r="E24" s="4"/>
-      <c r="F24" s="4"/>
-      <c r="G24" s="4"/>
-      <c r="H24" s="4"/>
-      <c r="I24" s="6"/>
-      <c r="J24" s="6"/>
+    <row r="24" ht="304.5" spans="1:10">
+      <c r="A24" s="6" t="s">
+        <v>124</v>
+      </c>
+      <c r="B24" s="6" t="s">
+        <v>125</v>
+      </c>
+      <c r="C24" s="6" t="s">
+        <v>126</v>
+      </c>
+      <c r="D24" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="E24" s="6">
+        <v>1</v>
+      </c>
+      <c r="F24" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="G24" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="H24" s="6" t="s">
+        <v>128</v>
+      </c>
+      <c r="I24" s="7">
+        <v>46101</v>
+      </c>
+      <c r="J24" s="7">
+        <v>46107</v>
+      </c>
     </row>
-    <row r="25" ht="14.5" spans="1:10">
-      <c r="A25" s="4"/>
-      <c r="B25" s="4"/>
-      <c r="C25" s="4"/>
-      <c r="D25" s="4"/>
-      <c r="E25" s="4"/>
-      <c r="F25" s="4"/>
-      <c r="G25" s="4"/>
-      <c r="H25" s="4"/>
-      <c r="I25" s="6"/>
-      <c r="J25" s="6"/>
+    <row r="25" ht="409.5" spans="1:10">
+      <c r="A25" s="6" t="s">
+        <v>129</v>
+      </c>
+      <c r="B25" s="6" t="s">
+        <v>130</v>
+      </c>
+      <c r="C25" s="6" t="s">
+        <v>131</v>
+      </c>
+      <c r="D25" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="E25" s="6">
+        <v>1</v>
+      </c>
+      <c r="F25" s="6" t="s">
+        <v>132</v>
+      </c>
+      <c r="G25" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="H25" s="6" t="s">
+        <v>133</v>
+      </c>
+      <c r="I25" s="7">
+        <v>46108</v>
+      </c>
+      <c r="J25" s="7">
+        <v>46112</v>
+      </c>
     </row>
-    <row r="26" ht="14.5" spans="1:10">
-      <c r="A26" s="4"/>
-      <c r="B26" s="4"/>
-      <c r="C26" s="4"/>
-      <c r="D26" s="4"/>
-      <c r="E26" s="4"/>
-      <c r="F26" s="4"/>
-      <c r="G26" s="4"/>
-      <c r="H26" s="4"/>
-      <c r="I26" s="6"/>
-      <c r="J26" s="6"/>
-    </row>
-    <row r="27" ht="14.5" spans="1:10">
-      <c r="A27" s="4"/>
-      <c r="B27" s="4"/>
-      <c r="C27" s="4"/>
-      <c r="D27" s="4"/>
-      <c r="E27" s="4"/>
-      <c r="F27" s="4"/>
-      <c r="G27" s="4"/>
-      <c r="H27" s="4"/>
-      <c r="I27" s="6"/>
-      <c r="J27" s="6"/>
+    <row r="26" ht="391.5" spans="1:10">
+      <c r="A26" s="6" t="s">
+        <v>134</v>
+      </c>
+      <c r="B26" s="6" t="s">
+        <v>135</v>
+      </c>
+      <c r="C26" s="6" t="s">
+        <v>136</v>
+      </c>
+      <c r="D26" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="E26" s="6">
+        <v>1</v>
+      </c>
+      <c r="F26" s="6" t="s">
+        <v>137</v>
+      </c>
+      <c r="G26" s="6" t="s">
+        <v>138</v>
+      </c>
+      <c r="H26" s="6" t="s">
+        <v>139</v>
+      </c>
+      <c r="I26" s="7">
+        <v>46113</v>
+      </c>
+      <c r="J26" s="7">
+        <v>46119</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
[Stage 1] Update prioritisation
</commit_message>
<xml_diff>
--- a/product backlog template.xlsx
+++ b/product backlog template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\software_engineering\software-engineering\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF6175D2-CDA7-4D4B-A7CC-1593E8824A38}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{03E0053A-B24E-4EA2-BD94-8BD1E1750F64}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="121">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="123">
   <si>
     <t>Story ID</t>
   </si>
@@ -93,9 +93,6 @@
 So that it complies with the rule "TAs can take at most 3 courses at the same time", no need to count workload, and directly control the registration limit</t>
   </si>
   <si>
-    <t>High</t>
-  </si>
-  <si>
     <t>1. The system automatically counts the number of course TA positions each TA currently holds, and marks "Reached Upper Limit" when the number = 3
 2. When marked TAs register for new positions, the system pops up a prompt "Already holds 3 courses, cannot register for new positions" and blocks the registration operation
 3. In the administrator page list, the names of TAs "Reached Upper Limit" are highlighted in red, with a note "Currently 3 courses"
@@ -138,9 +135,6 @@
 So that the risk of "creating accounts first and then reviewing" is avoided, and only MOs recognized by the school can obtain system access rights</t>
   </si>
   <si>
-    <t>Medium</t>
-  </si>
-  <si>
     <r>
       <rPr>
         <sz val="11"/>
@@ -466,9 +460,6 @@
       </rPr>
       <t>So that stop irregular operations in time, prevent system data from being tampered with, and ensure the order of system use and data security</t>
     </r>
-  </si>
-  <si>
-    <t>low</t>
   </si>
   <si>
     <r>
@@ -754,10 +745,6 @@
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
   <si>
-    <t>High</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
     <t>As a TA applicant, I want to provide a dedicated application statement when applying for a specific TA position, so that I can have a further communication with the MO.</t>
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
@@ -769,6 +756,27 @@
   </si>
   <si>
     <t>Provide applicants with an additional channel for in-depth communication with instructors, helping the MO better understand the applicant’s motivation, strengths and fit for the role.</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>Must have</t>
+  </si>
+  <si>
+    <t>Must have</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>Should have</t>
+  </si>
+  <si>
+    <t>Should have</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>Could have</t>
+  </si>
+  <si>
+    <t>Could have</t>
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
 </sst>
@@ -1241,19 +1249,19 @@
         <v>15</v>
       </c>
       <c r="D3" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="E3" s="3">
+        <v>1</v>
+      </c>
+      <c r="F3" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="E3" s="3">
-        <v>1</v>
-      </c>
-      <c r="F3" s="3" t="s">
+      <c r="G3" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="G3" s="3" t="s">
+      <c r="H3" s="3" t="s">
         <v>18</v>
-      </c>
-      <c r="H3" s="3" t="s">
-        <v>19</v>
       </c>
       <c r="I3" s="4">
         <v>46101</v>
@@ -1264,28 +1272,28 @@
     </row>
     <row r="4" spans="1:10" ht="377" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B4" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="C4" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="D4" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="E4" s="3">
+        <v>1</v>
+      </c>
+      <c r="F4" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="D4" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="E4" s="3">
-        <v>1</v>
-      </c>
-      <c r="F4" s="3" t="s">
+      <c r="G4" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="H4" s="3" t="s">
         <v>23</v>
-      </c>
-      <c r="G4" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="H4" s="3" t="s">
-        <v>24</v>
       </c>
       <c r="I4" s="4">
         <v>46124</v>
@@ -1296,28 +1304,28 @@
     </row>
     <row r="5" spans="1:10" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="B5" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="C5" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="D5" s="3" t="s">
+        <v>120</v>
+      </c>
+      <c r="E5" s="3">
+        <v>1</v>
+      </c>
+      <c r="F5" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="G5" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="E5" s="3">
-        <v>1</v>
-      </c>
-      <c r="F5" s="3" t="s">
+      <c r="H5" s="3" t="s">
         <v>29</v>
-      </c>
-      <c r="G5" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="H5" s="3" t="s">
-        <v>31</v>
       </c>
       <c r="I5" s="4">
         <v>46108</v>
@@ -1328,28 +1336,28 @@
     </row>
     <row r="6" spans="1:10" ht="217.5" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="C6" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="D6" s="3" t="s">
+        <v>119</v>
+      </c>
+      <c r="E6" s="3">
+        <v>1</v>
+      </c>
+      <c r="F6" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="C6" s="3" t="s">
+      <c r="G6" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="D6" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="E6" s="3">
-        <v>1</v>
-      </c>
-      <c r="F6" s="3" t="s">
+      <c r="H6" s="3" t="s">
         <v>35</v>
-      </c>
-      <c r="G6" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="H6" s="3" t="s">
-        <v>37</v>
       </c>
       <c r="I6" s="4">
         <v>46108</v>
@@ -1360,28 +1368,28 @@
     </row>
     <row r="7" spans="1:10" ht="333.5" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="C7" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="D7" s="3" t="s">
+        <v>119</v>
+      </c>
+      <c r="E7" s="3">
+        <v>1</v>
+      </c>
+      <c r="F7" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="C7" s="3" t="s">
+      <c r="G7" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="H7" s="3" t="s">
         <v>40</v>
-      </c>
-      <c r="D7" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="E7" s="3">
-        <v>1</v>
-      </c>
-      <c r="F7" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="G7" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="H7" s="3" t="s">
-        <v>42</v>
       </c>
       <c r="I7" s="4">
         <v>46113</v>
@@ -1392,28 +1400,28 @@
     </row>
     <row r="8" spans="1:10" ht="217.5" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="C8" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="B8" s="3" t="s">
+      <c r="D8" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="E8" s="3">
+        <v>1</v>
+      </c>
+      <c r="F8" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="C8" s="3" t="s">
+      <c r="G8" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="H8" s="3" t="s">
         <v>45</v>
-      </c>
-      <c r="D8" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="E8" s="3">
-        <v>1</v>
-      </c>
-      <c r="F8" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="G8" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="H8" s="3" t="s">
-        <v>48</v>
       </c>
       <c r="I8" s="4">
         <v>46119</v>
@@ -1424,28 +1432,28 @@
     </row>
     <row r="9" spans="1:10" ht="174" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="E9" s="3">
+        <v>1</v>
+      </c>
+      <c r="F9" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="G9" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="B9" s="3" t="s">
+      <c r="H9" s="3" t="s">
         <v>50</v>
-      </c>
-      <c r="C9" s="3" t="s">
-        <v>109</v>
-      </c>
-      <c r="D9" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="E9" s="3">
-        <v>1</v>
-      </c>
-      <c r="F9" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="G9" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="H9" s="3" t="s">
-        <v>53</v>
       </c>
       <c r="I9" s="5">
         <v>46101</v>
@@ -1456,28 +1464,28 @@
     </row>
     <row r="10" spans="1:10" ht="130.5" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="E10" s="3">
+        <v>1</v>
+      </c>
+      <c r="F10" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="G10" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="H10" s="3" t="s">
         <v>54</v>
-      </c>
-      <c r="B10" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="C10" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="D10" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="E10" s="3">
-        <v>1</v>
-      </c>
-      <c r="F10" s="3" t="s">
-        <v>110</v>
-      </c>
-      <c r="G10" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="H10" s="3" t="s">
-        <v>57</v>
       </c>
       <c r="I10" s="5">
         <v>46101</v>
@@ -1488,28 +1496,28 @@
     </row>
     <row r="11" spans="1:10" ht="116" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="E11" s="3">
+        <v>1</v>
+      </c>
+      <c r="F11" s="3" t="s">
+        <v>108</v>
+      </c>
+      <c r="G11" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="H11" s="3" t="s">
         <v>58</v>
-      </c>
-      <c r="B11" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="C11" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="D11" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="E11" s="3">
-        <v>1</v>
-      </c>
-      <c r="F11" s="3" t="s">
-        <v>111</v>
-      </c>
-      <c r="G11" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="H11" s="3" t="s">
-        <v>61</v>
       </c>
       <c r="I11" s="5">
         <v>46101</v>
@@ -1520,28 +1528,28 @@
     </row>
     <row r="12" spans="1:10" ht="145" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="D12" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="E12" s="3">
+        <v>1</v>
+      </c>
+      <c r="F12" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="B12" s="3" t="s">
+      <c r="G12" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="H12" s="3" t="s">
         <v>63</v>
-      </c>
-      <c r="C12" s="3" t="s">
-        <v>64</v>
-      </c>
-      <c r="D12" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="E12" s="3">
-        <v>1</v>
-      </c>
-      <c r="F12" s="3" t="s">
-        <v>65</v>
-      </c>
-      <c r="G12" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="H12" s="3" t="s">
-        <v>66</v>
       </c>
       <c r="I12" s="5">
         <v>46101</v>
@@ -1552,13 +1560,13 @@
     </row>
     <row r="13" spans="1:10" ht="174" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="D13" s="3" t="s">
         <v>117</v>
@@ -1567,13 +1575,13 @@
         <v>1</v>
       </c>
       <c r="F13" s="3" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="G13" s="3" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="H13" s="3" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="I13" s="5">
         <v>46113</v>
@@ -1584,28 +1592,28 @@
     </row>
     <row r="14" spans="1:10" ht="159.5" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="D14" s="3" t="s">
+        <v>119</v>
+      </c>
+      <c r="E14" s="3">
+        <v>1</v>
+      </c>
+      <c r="F14" s="3" t="s">
+        <v>111</v>
+      </c>
+      <c r="G14" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="E14" s="3">
-        <v>1</v>
-      </c>
-      <c r="F14" s="3" t="s">
-        <v>114</v>
-      </c>
-      <c r="G14" s="3" t="s">
-        <v>30</v>
-      </c>
       <c r="H14" s="3" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="I14" s="5">
         <v>46108</v>
@@ -1616,28 +1624,28 @@
     </row>
     <row r="15" spans="1:10" ht="145" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="B15" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="C15" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="D15" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="E15" s="3">
+        <v>1</v>
+      </c>
+      <c r="F15" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="G15" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="H15" s="3" t="s">
         <v>68</v>
-      </c>
-      <c r="C15" s="3" t="s">
-        <v>69</v>
-      </c>
-      <c r="D15" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="E15" s="3">
-        <v>1</v>
-      </c>
-      <c r="F15" s="3" t="s">
-        <v>70</v>
-      </c>
-      <c r="G15" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="H15" s="3" t="s">
-        <v>71</v>
       </c>
       <c r="I15" s="5">
         <v>46113</v>
@@ -1648,28 +1656,28 @@
     </row>
     <row r="16" spans="1:10" ht="116" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="B16" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="C16" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="D16" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="E16" s="3">
+        <v>1</v>
+      </c>
+      <c r="F16" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="G16" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="H16" s="3" t="s">
         <v>72</v>
-      </c>
-      <c r="C16" s="3" t="s">
-        <v>73</v>
-      </c>
-      <c r="D16" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="E16" s="3">
-        <v>1</v>
-      </c>
-      <c r="F16" s="3" t="s">
-        <v>74</v>
-      </c>
-      <c r="G16" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="H16" s="3" t="s">
-        <v>75</v>
       </c>
       <c r="I16" s="5">
         <v>46113</v>
@@ -1680,28 +1688,28 @@
     </row>
     <row r="17" spans="1:10" ht="101.5" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="B17" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="D17" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="E17" s="3">
+        <v>1</v>
+      </c>
+      <c r="F17" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="G17" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="H17" s="3" t="s">
         <v>76</v>
-      </c>
-      <c r="C17" s="3" t="s">
-        <v>77</v>
-      </c>
-      <c r="D17" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="E17" s="3">
-        <v>1</v>
-      </c>
-      <c r="F17" s="3" t="s">
-        <v>78</v>
-      </c>
-      <c r="G17" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="H17" s="3" t="s">
-        <v>79</v>
       </c>
       <c r="I17" s="5">
         <v>46113</v>
@@ -1712,28 +1720,28 @@
     </row>
     <row r="18" spans="1:10" ht="319" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="C18" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="D18" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="E18" s="3">
+        <v>1</v>
+      </c>
+      <c r="F18" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="B18" s="3" t="s">
+      <c r="G18" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="H18" s="3" t="s">
         <v>81</v>
-      </c>
-      <c r="C18" s="3" t="s">
-        <v>82</v>
-      </c>
-      <c r="D18" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="E18" s="3">
-        <v>1</v>
-      </c>
-      <c r="F18" s="3" t="s">
-        <v>83</v>
-      </c>
-      <c r="G18" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="H18" s="3" t="s">
-        <v>84</v>
       </c>
       <c r="I18" s="5">
         <v>46101</v>
@@ -1744,28 +1752,28 @@
     </row>
     <row r="19" spans="1:10" ht="304.5" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="C19" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="D19" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="E19" s="3">
+        <v>1</v>
+      </c>
+      <c r="F19" s="3" t="s">
         <v>85</v>
       </c>
-      <c r="B19" s="3" t="s">
+      <c r="G19" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="H19" s="3" t="s">
         <v>86</v>
-      </c>
-      <c r="C19" s="3" t="s">
-        <v>87</v>
-      </c>
-      <c r="D19" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="E19" s="3">
-        <v>1</v>
-      </c>
-      <c r="F19" s="3" t="s">
-        <v>88</v>
-      </c>
-      <c r="G19" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="H19" s="3" t="s">
-        <v>89</v>
       </c>
       <c r="I19" s="5">
         <v>46101</v>
@@ -1776,28 +1784,28 @@
     </row>
     <row r="20" spans="1:10" ht="304.5" x14ac:dyDescent="0.25">
       <c r="A20" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="C20" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="D20" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="E20" s="3">
+        <v>1</v>
+      </c>
+      <c r="F20" s="3" t="s">
         <v>90</v>
       </c>
-      <c r="B20" s="3" t="s">
+      <c r="G20" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="H20" s="3" t="s">
         <v>91</v>
-      </c>
-      <c r="C20" s="3" t="s">
-        <v>92</v>
-      </c>
-      <c r="D20" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="E20" s="3">
-        <v>1</v>
-      </c>
-      <c r="F20" s="3" t="s">
-        <v>93</v>
-      </c>
-      <c r="G20" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="H20" s="3" t="s">
-        <v>94</v>
       </c>
       <c r="I20" s="5">
         <v>46101</v>
@@ -1808,28 +1816,28 @@
     </row>
     <row r="21" spans="1:10" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A21" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="C21" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="D21" s="3" t="s">
+        <v>119</v>
+      </c>
+      <c r="E21" s="3">
+        <v>1</v>
+      </c>
+      <c r="F21" s="3" t="s">
         <v>95</v>
       </c>
-      <c r="B21" s="3" t="s">
+      <c r="G21" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="H21" s="3" t="s">
         <v>96</v>
-      </c>
-      <c r="C21" s="3" t="s">
-        <v>97</v>
-      </c>
-      <c r="D21" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="E21" s="3">
-        <v>1</v>
-      </c>
-      <c r="F21" s="3" t="s">
-        <v>98</v>
-      </c>
-      <c r="G21" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="H21" s="3" t="s">
-        <v>99</v>
       </c>
       <c r="I21" s="5">
         <v>46108</v>
@@ -1840,28 +1848,28 @@
     </row>
     <row r="22" spans="1:10" ht="391.5" x14ac:dyDescent="0.25">
       <c r="A22" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="B22" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="C22" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="D22" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="E22" s="3">
+        <v>1</v>
+      </c>
+      <c r="F22" s="3" t="s">
         <v>100</v>
       </c>
-      <c r="B22" s="3" t="s">
+      <c r="G22" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="H22" s="3" t="s">
         <v>101</v>
-      </c>
-      <c r="C22" s="3" t="s">
-        <v>102</v>
-      </c>
-      <c r="D22" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="E22" s="3">
-        <v>1</v>
-      </c>
-      <c r="F22" s="3" t="s">
-        <v>103</v>
-      </c>
-      <c r="G22" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="H22" s="3" t="s">
-        <v>104</v>
       </c>
       <c r="I22" s="5">
         <v>46113</v>

</xml_diff>

<commit_message>
[Stage 1] Update backlog
</commit_message>
<xml_diff>
--- a/product backlog template.xlsx
+++ b/product backlog template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\software_engineering\software-engineering\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{03E0053A-B24E-4EA2-BD94-8BD1E1750F64}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE1D8ED8-66BE-4324-B1B4-E3E880082568}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="123">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="117">
   <si>
     <t>Story ID</t>
   </si>
@@ -124,25 +124,20 @@
     <t>Optimize the TA recruitment process, realize efficient linkage between administrators and MOs               (Priority raised to High according to teacher's suggestions, core linkage function)</t>
   </si>
   <si>
-    <t>AD003</t>
-  </si>
-  <si>
-    <t>Review MO Self-Registered Accounts (Verify Identity Synchronously During Registration)</t>
-  </si>
-  <si>
-    <t>As a system admin
-I want to verify MOs' identities (such as employment certificates) synchronously when they submit account registration applications, and only create MO accounts after approval
-So that the risk of "creating accounts first and then reviewing" is avoided, and only MOs recognized by the school can obtain system access rights</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>1. The system has a dedicated "MO Permission Review" page, with pending applications ranked first and highlighted in red as a reminder</t>
+    <t>2 story points</t>
+  </si>
+  <si>
+    <t>Batch Import/Export TA Basic Information</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>As a system admin</t>
     </r>
     <r>
       <rPr>
@@ -161,7 +156,7 @@
         <rFont val="Calibri"/>
         <family val="2"/>
       </rPr>
-      <t>2. The application card displays the MO's name, department, specific applied permissions and uploaded employment certification materials</t>
+      <t>I want to batch import TA basic information via CSV files and export all TA information as CSV files with one click</t>
     </r>
     <r>
       <rPr>
@@ -180,7 +175,18 @@
         <rFont val="Calibri"/>
         <family val="2"/>
       </rPr>
-      <t>3. Review operations: Click "Approve" and the MO will obtain the corresponding permissions immediately; click "Reject" to enter the reason, which can be viewed by the MO after logging in</t>
+      <t>So that there is no need to create TA accounts one by one, improve work efficiency, and facilitate backing up TA data or submitting it to the school for filing</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>1. Batch export: Export all TA information with one click, including account status and basic information, the file format meets the requirements of plain text</t>
     </r>
     <r>
       <rPr>
@@ -199,20 +205,17 @@
         <rFont val="Calibri"/>
         <family val="2"/>
       </rPr>
-      <t>4. After the review is completed, the application is automatically classified into the "Approved/Rejected" list, supporting filtering by name/review status</t>
-    </r>
-  </si>
-  <si>
-    <t>2 story points</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dependent on the MO-side permission application function                        </t>
-  </si>
-  <si>
-    <t>AD004</t>
-  </si>
-  <si>
-    <t>Batch Import/Export TA Basic Information</t>
+      <t>2. Export filter: Support filtering by account status (Active/Deactivated) and export only the TA information that meets the conditions</t>
+    </r>
+  </si>
+  <si>
+    <t>1 story points</t>
+  </si>
+  <si>
+    <t>maybe "export"is more needed</t>
+  </si>
+  <si>
+    <t>View All System Operation Records with CSV Export Function</t>
   </si>
   <si>
     <r>
@@ -241,7 +244,7 @@
         <rFont val="Calibri"/>
         <family val="2"/>
       </rPr>
-      <t>I want to batch import TA basic information via CSV files and export all TA information as CSV files with one click</t>
+      <t>I want to view all operations of TAs, MOs and other admins in the system, and export the filtered records as CSV files to the computer</t>
     </r>
     <r>
       <rPr>
@@ -260,18 +263,18 @@
         <rFont val="Calibri"/>
         <family val="2"/>
       </rPr>
-      <t>So that there is no need to create TA accounts one by one, improve work efficiency, and facilitate backing up TA data or submitting it to the school for filing</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>1. Batch export: Export all TA information with one click, including account status and basic information, the file format meets the requirements of plain text</t>
+      <t>So that I can accurately trace who performed irregular operations (e.g., modifying tasks, deleting information) and when</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>1. Operation records include: operator, account type (TA/MO/Admin), operation type, operation time, operation content and operation result</t>
     </r>
     <r>
       <rPr>
@@ -290,30 +293,7 @@
         <rFont val="Calibri"/>
         <family val="2"/>
       </rPr>
-      <t>2. Export filter: Support filtering by account status (Active/Deactivated) and export only the TA information that meets the conditions</t>
-    </r>
-  </si>
-  <si>
-    <t>1 story points</t>
-  </si>
-  <si>
-    <t>maybe "export"is more needed</t>
-  </si>
-  <si>
-    <t>AD005</t>
-  </si>
-  <si>
-    <t>View All System Operation Records with CSV Export Function</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>As a system admin</t>
+      <t>2. Support multi-condition combined filtering: filter by account type, operation type and time range, with one-click refresh of results</t>
     </r>
     <r>
       <rPr>
@@ -332,82 +312,11 @@
         <rFont val="Calibri"/>
         <family val="2"/>
       </rPr>
-      <t>I want to view all operations of TAs, MOs and other admins in the system, and export the filtered records as CSV files to the computer</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>So that I can accurately trace who performed irregular operations (e.g., modifying tasks, deleting information) and when</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>1. Operation records include: operator, account type (TA/MO/Admin), operation type, operation time, operation content and operation result</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>2. Support multi-condition combined filtering: filter by account type, operation type and time range, with one-click refresh of results</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
       <t>3. Export function: Click "Export CSV" and the file is downloaded directly to the computer, the format meets the project's plain text requirements</t>
     </r>
   </si>
   <si>
     <t>Necessary function for system security, non-core but mandatory, to be developed and completed in Sprint 3</t>
-  </si>
-  <si>
-    <t>AD006</t>
   </si>
   <si>
     <t>Quickly Freeze Abnormal TA/MO Accounts</t>
@@ -769,14 +678,22 @@
     <t>Should have</t>
   </si>
   <si>
-    <t>Should have</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
     <t>Could have</t>
   </si>
   <si>
     <t>Could have</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>AD003</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>AD004</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>AD005</t>
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
 </sst>
@@ -1181,7 +1098,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J22"/>
+  <dimension ref="A1:J21"/>
   <sheetFormatPr defaultColWidth="8.90625" defaultRowHeight="14" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.08984375" style="1" customWidth="1"/>
@@ -1249,7 +1166,7 @@
         <v>15</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>118</v>
+        <v>110</v>
       </c>
       <c r="E3" s="3">
         <v>1</v>
@@ -1281,7 +1198,7 @@
         <v>21</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>117</v>
+        <v>109</v>
       </c>
       <c r="E4" s="3">
         <v>1</v>
@@ -1302,9 +1219,9 @@
         <v>46132</v>
       </c>
     </row>
-    <row r="5" spans="1:10" ht="409.5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:10" ht="217.5" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>24</v>
+        <v>114</v>
       </c>
       <c r="B5" s="3" t="s">
         <v>25</v>
@@ -1313,7 +1230,7 @@
         <v>26</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>120</v>
+        <v>111</v>
       </c>
       <c r="E5" s="3">
         <v>1</v>
@@ -1334,126 +1251,126 @@
         <v>46112</v>
       </c>
     </row>
-    <row r="6" spans="1:10" ht="217.5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:10" ht="333.5" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="B6" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="C6" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="C6" s="3" t="s">
+      <c r="D6" s="3" t="s">
+        <v>111</v>
+      </c>
+      <c r="E6" s="3">
+        <v>1</v>
+      </c>
+      <c r="F6" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="D6" s="3" t="s">
-        <v>119</v>
-      </c>
-      <c r="E6" s="3">
-        <v>1</v>
-      </c>
-      <c r="F6" s="3" t="s">
+      <c r="G6" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="H6" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="G6" s="3" t="s">
+      <c r="I6" s="4">
+        <v>46113</v>
+      </c>
+      <c r="J6" s="4">
+        <v>46118</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" ht="217.5" x14ac:dyDescent="0.25">
+      <c r="A7" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="B7" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="H6" s="3" t="s">
+      <c r="C7" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="I6" s="4">
-        <v>46108</v>
-      </c>
-      <c r="J6" s="4">
-        <v>46112</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10" ht="333.5" x14ac:dyDescent="0.25">
-      <c r="A7" s="3" t="s">
+      <c r="D7" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="E7" s="3">
+        <v>1</v>
+      </c>
+      <c r="F7" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="G7" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="H7" s="3" t="s">
         <v>37</v>
       </c>
-      <c r="C7" s="3" t="s">
+      <c r="I7" s="4">
+        <v>46119</v>
+      </c>
+      <c r="J7" s="4">
+        <v>46124</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" ht="174" x14ac:dyDescent="0.25">
+      <c r="A8" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="D7" s="3" t="s">
-        <v>119</v>
-      </c>
-      <c r="E7" s="3">
-        <v>1</v>
-      </c>
-      <c r="F7" s="3" t="s">
+      <c r="B8" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="G7" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="H7" s="3" t="s">
+      <c r="C8" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="E8" s="3">
+        <v>1</v>
+      </c>
+      <c r="F8" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="I7" s="4">
-        <v>46113</v>
-      </c>
-      <c r="J7" s="4">
-        <v>46118</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10" ht="217.5" x14ac:dyDescent="0.25">
-      <c r="A8" s="3" t="s">
+      <c r="G8" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="B8" s="3" t="s">
+      <c r="H8" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="C8" s="3" t="s">
+      <c r="I8" s="5">
+        <v>46101</v>
+      </c>
+      <c r="J8" s="5">
+        <v>46107</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" ht="130.5" x14ac:dyDescent="0.25">
+      <c r="A9" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="D8" s="3" t="s">
-        <v>122</v>
-      </c>
-      <c r="E8" s="3">
-        <v>1</v>
-      </c>
-      <c r="F8" s="3" t="s">
+      <c r="B9" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="G8" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="H8" s="3" t="s">
+      <c r="C9" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="I8" s="4">
-        <v>46119</v>
-      </c>
-      <c r="J8" s="4">
-        <v>46124</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10" ht="174" x14ac:dyDescent="0.25">
-      <c r="A9" s="3" t="s">
+      <c r="D9" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="E9" s="3">
+        <v>1</v>
+      </c>
+      <c r="F9" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="G9" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="H9" s="3" t="s">
         <v>46</v>
-      </c>
-      <c r="B9" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="C9" s="3" t="s">
-        <v>106</v>
-      </c>
-      <c r="D9" s="3" t="s">
-        <v>117</v>
-      </c>
-      <c r="E9" s="3">
-        <v>1</v>
-      </c>
-      <c r="F9" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="G9" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="H9" s="3" t="s">
-        <v>50</v>
       </c>
       <c r="I9" s="5">
         <v>46101</v>
@@ -1462,30 +1379,30 @@
         <v>46107</v>
       </c>
     </row>
-    <row r="10" spans="1:10" ht="130.5" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:10" ht="116" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>117</v>
+        <v>109</v>
       </c>
       <c r="E10" s="3">
         <v>1</v>
       </c>
       <c r="F10" s="3" t="s">
-        <v>107</v>
+        <v>100</v>
       </c>
       <c r="G10" s="3" t="s">
         <v>17</v>
       </c>
       <c r="H10" s="3" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="I10" s="5">
         <v>46101</v>
@@ -1494,30 +1411,30 @@
         <v>46107</v>
       </c>
     </row>
-    <row r="11" spans="1:10" ht="116" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:10" ht="145" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>117</v>
+        <v>109</v>
       </c>
       <c r="E11" s="3">
         <v>1</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>108</v>
+        <v>54</v>
       </c>
       <c r="G11" s="3" t="s">
         <v>17</v>
       </c>
       <c r="H11" s="3" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="I11" s="5">
         <v>46101</v>
@@ -1526,126 +1443,126 @@
         <v>46107</v>
       </c>
     </row>
-    <row r="12" spans="1:10" ht="145" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:10" ht="174" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="D12" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="E12" s="3">
+        <v>1</v>
+      </c>
+      <c r="F12" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="G12" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="H12" s="3" t="s">
+        <v>108</v>
+      </c>
+      <c r="I12" s="5">
+        <v>46113</v>
+      </c>
+      <c r="J12" s="5">
+        <v>46119</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" ht="159.5" x14ac:dyDescent="0.25">
+      <c r="A13" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="D13" s="3" t="s">
+        <v>111</v>
+      </c>
+      <c r="E13" s="3">
+        <v>1</v>
+      </c>
+      <c r="F13" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="G13" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="H13" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="I13" s="5">
+        <v>46108</v>
+      </c>
+      <c r="J13" s="5">
+        <v>46112</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" ht="145" x14ac:dyDescent="0.25">
+      <c r="A14" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="D14" s="3" t="s">
+        <v>112</v>
+      </c>
+      <c r="E14" s="3">
+        <v>1</v>
+      </c>
+      <c r="F14" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="B12" s="3" t="s">
+      <c r="G14" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="H14" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="C12" s="3" t="s">
+      <c r="I14" s="5">
+        <v>46113</v>
+      </c>
+      <c r="J14" s="5">
+        <v>46119</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" ht="116" x14ac:dyDescent="0.25">
+      <c r="A15" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="B15" s="3" t="s">
         <v>61</v>
       </c>
-      <c r="D12" s="3" t="s">
-        <v>117</v>
-      </c>
-      <c r="E12" s="3">
-        <v>1</v>
-      </c>
-      <c r="F12" s="3" t="s">
+      <c r="C15" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="G12" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="H12" s="3" t="s">
+      <c r="D15" s="3" t="s">
+        <v>112</v>
+      </c>
+      <c r="E15" s="3">
+        <v>1</v>
+      </c>
+      <c r="F15" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="I12" s="5">
-        <v>46101</v>
-      </c>
-      <c r="J12" s="5">
-        <v>46107</v>
-      </c>
-    </row>
-    <row r="13" spans="1:10" ht="174" x14ac:dyDescent="0.25">
-      <c r="A13" s="3" t="s">
-        <v>102</v>
-      </c>
-      <c r="B13" s="3" t="s">
-        <v>113</v>
-      </c>
-      <c r="C13" s="3" t="s">
-        <v>114</v>
-      </c>
-      <c r="D13" s="3" t="s">
-        <v>117</v>
-      </c>
-      <c r="E13" s="3">
-        <v>1</v>
-      </c>
-      <c r="F13" s="3" t="s">
-        <v>115</v>
-      </c>
-      <c r="G13" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="H13" s="3" t="s">
-        <v>116</v>
-      </c>
-      <c r="I13" s="5">
-        <v>46113</v>
-      </c>
-      <c r="J13" s="5">
-        <v>46119</v>
-      </c>
-    </row>
-    <row r="14" spans="1:10" ht="159.5" x14ac:dyDescent="0.25">
-      <c r="A14" s="3" t="s">
-        <v>103</v>
-      </c>
-      <c r="B14" s="3" t="s">
-        <v>109</v>
-      </c>
-      <c r="C14" s="3" t="s">
-        <v>110</v>
-      </c>
-      <c r="D14" s="3" t="s">
-        <v>119</v>
-      </c>
-      <c r="E14" s="3">
-        <v>1</v>
-      </c>
-      <c r="F14" s="3" t="s">
-        <v>111</v>
-      </c>
-      <c r="G14" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="H14" s="3" t="s">
+      <c r="G15" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="H15" s="3" t="s">
         <v>64</v>
-      </c>
-      <c r="I14" s="5">
-        <v>46108</v>
-      </c>
-      <c r="J14" s="5">
-        <v>46112</v>
-      </c>
-    </row>
-    <row r="15" spans="1:10" ht="145" x14ac:dyDescent="0.25">
-      <c r="A15" s="3" t="s">
-        <v>104</v>
-      </c>
-      <c r="B15" s="3" t="s">
-        <v>65</v>
-      </c>
-      <c r="C15" s="3" t="s">
-        <v>66</v>
-      </c>
-      <c r="D15" s="3" t="s">
-        <v>121</v>
-      </c>
-      <c r="E15" s="3">
-        <v>1</v>
-      </c>
-      <c r="F15" s="3" t="s">
-        <v>67</v>
-      </c>
-      <c r="G15" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="H15" s="3" t="s">
-        <v>68</v>
       </c>
       <c r="I15" s="5">
         <v>46113</v>
@@ -1654,30 +1571,30 @@
         <v>46119</v>
       </c>
     </row>
-    <row r="16" spans="1:10" ht="116" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:10" ht="101.5" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>121</v>
+        <v>112</v>
       </c>
       <c r="E16" s="3">
         <v>1</v>
       </c>
       <c r="F16" s="3" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="G16" s="3" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="H16" s="3" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="I16" s="5">
         <v>46113</v>
@@ -1686,62 +1603,62 @@
         <v>46119</v>
       </c>
     </row>
-    <row r="17" spans="1:10" ht="101.5" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:10" ht="319" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
-        <v>112</v>
+        <v>69</v>
       </c>
       <c r="B17" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="D17" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="E17" s="3">
+        <v>1</v>
+      </c>
+      <c r="F17" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="G17" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="H17" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="C17" s="3" t="s">
+      <c r="I17" s="5">
+        <v>46101</v>
+      </c>
+      <c r="J17" s="5">
+        <v>46107</v>
+      </c>
+    </row>
+    <row r="18" spans="1:10" ht="304.5" x14ac:dyDescent="0.25">
+      <c r="A18" s="3" t="s">
         <v>74</v>
       </c>
-      <c r="D17" s="3" t="s">
-        <v>121</v>
-      </c>
-      <c r="E17" s="3">
-        <v>1</v>
-      </c>
-      <c r="F17" s="3" t="s">
+      <c r="B18" s="3" t="s">
         <v>75</v>
       </c>
-      <c r="G17" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="H17" s="3" t="s">
+      <c r="C18" s="3" t="s">
         <v>76</v>
       </c>
-      <c r="I17" s="5">
-        <v>46113</v>
-      </c>
-      <c r="J17" s="5">
-        <v>46119</v>
-      </c>
-    </row>
-    <row r="18" spans="1:10" ht="319" x14ac:dyDescent="0.25">
-      <c r="A18" s="3" t="s">
+      <c r="D18" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="E18" s="3">
+        <v>1</v>
+      </c>
+      <c r="F18" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="B18" s="3" t="s">
+      <c r="G18" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="H18" s="3" t="s">
         <v>78</v>
-      </c>
-      <c r="C18" s="3" t="s">
-        <v>79</v>
-      </c>
-      <c r="D18" s="3" t="s">
-        <v>117</v>
-      </c>
-      <c r="E18" s="3">
-        <v>1</v>
-      </c>
-      <c r="F18" s="3" t="s">
-        <v>80</v>
-      </c>
-      <c r="G18" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="H18" s="3" t="s">
-        <v>81</v>
       </c>
       <c r="I18" s="5">
         <v>46101</v>
@@ -1752,28 +1669,28 @@
     </row>
     <row r="19" spans="1:10" ht="304.5" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="C19" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="D19" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="E19" s="3">
+        <v>1</v>
+      </c>
+      <c r="F19" s="3" t="s">
         <v>82</v>
       </c>
-      <c r="B19" s="3" t="s">
+      <c r="G19" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="H19" s="3" t="s">
         <v>83</v>
-      </c>
-      <c r="C19" s="3" t="s">
-        <v>84</v>
-      </c>
-      <c r="D19" s="3" t="s">
-        <v>117</v>
-      </c>
-      <c r="E19" s="3">
-        <v>1</v>
-      </c>
-      <c r="F19" s="3" t="s">
-        <v>85</v>
-      </c>
-      <c r="G19" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="H19" s="3" t="s">
-        <v>86</v>
       </c>
       <c r="I19" s="5">
         <v>46101</v>
@@ -1782,99 +1699,67 @@
         <v>46107</v>
       </c>
     </row>
-    <row r="20" spans="1:10" ht="304.5" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:10" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A20" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="C20" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="D20" s="3" t="s">
+        <v>111</v>
+      </c>
+      <c r="E20" s="3">
+        <v>1</v>
+      </c>
+      <c r="F20" s="3" t="s">
         <v>87</v>
       </c>
-      <c r="B20" s="3" t="s">
+      <c r="G20" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="H20" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="C20" s="3" t="s">
+      <c r="I20" s="5">
+        <v>46108</v>
+      </c>
+      <c r="J20" s="5">
+        <v>46112</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" ht="391.5" x14ac:dyDescent="0.25">
+      <c r="A21" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="D20" s="3" t="s">
-        <v>117</v>
-      </c>
-      <c r="E20" s="3">
-        <v>1</v>
-      </c>
-      <c r="F20" s="3" t="s">
+      <c r="B21" s="3" t="s">
         <v>90</v>
       </c>
-      <c r="G20" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="H20" s="3" t="s">
+      <c r="C21" s="3" t="s">
         <v>91</v>
       </c>
-      <c r="I20" s="5">
-        <v>46101</v>
-      </c>
-      <c r="J20" s="5">
-        <v>46107</v>
-      </c>
-    </row>
-    <row r="21" spans="1:10" ht="409.5" x14ac:dyDescent="0.25">
-      <c r="A21" s="3" t="s">
+      <c r="D21" s="3" t="s">
+        <v>112</v>
+      </c>
+      <c r="E21" s="3">
+        <v>1</v>
+      </c>
+      <c r="F21" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="B21" s="3" t="s">
+      <c r="G21" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="H21" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="C21" s="3" t="s">
-        <v>94</v>
-      </c>
-      <c r="D21" s="3" t="s">
-        <v>119</v>
-      </c>
-      <c r="E21" s="3">
-        <v>1</v>
-      </c>
-      <c r="F21" s="3" t="s">
-        <v>95</v>
-      </c>
-      <c r="G21" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="H21" s="3" t="s">
-        <v>96</v>
-      </c>
       <c r="I21" s="5">
-        <v>46108</v>
+        <v>46113</v>
       </c>
       <c r="J21" s="5">
-        <v>46112</v>
-      </c>
-    </row>
-    <row r="22" spans="1:10" ht="391.5" x14ac:dyDescent="0.25">
-      <c r="A22" s="3" t="s">
-        <v>97</v>
-      </c>
-      <c r="B22" s="3" t="s">
-        <v>98</v>
-      </c>
-      <c r="C22" s="3" t="s">
-        <v>99</v>
-      </c>
-      <c r="D22" s="3" t="s">
-        <v>121</v>
-      </c>
-      <c r="E22" s="3">
-        <v>1</v>
-      </c>
-      <c r="F22" s="3" t="s">
-        <v>100</v>
-      </c>
-      <c r="G22" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="H22" s="3" t="s">
-        <v>101</v>
-      </c>
-      <c r="I22" s="5">
-        <v>46113</v>
-      </c>
-      <c r="J22" s="5">
         <v>46119</v>
       </c>
     </row>

</xml_diff>